<commit_message>
feat: product images, alphabetical sort, contact info, QR share section, favicon
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="169" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="169" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\-mmm"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -85,6 +85,12 @@
       <name val="Arial"/>
       <charset val="204"/>
       <family val="2"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -151,7 +157,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -214,6 +220,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -479,19 +488,19 @@
   <dimension ref="A1:S179"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="23.77734375" customWidth="1" min="1" max="1"/>
     <col width="7.6640625" customWidth="1" min="2" max="2"/>
     <col width="9.33203125" customWidth="1" min="3" max="3"/>
     <col width="9.44140625" customWidth="1" min="4" max="4"/>
     <col width="7.21875" customWidth="1" min="5" max="5"/>
-    <col width="36" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="35.77734375" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="128.33203125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="25.21875" customWidth="1" min="6" max="6"/>
+    <col width="35.77734375" customWidth="1" min="7" max="7"/>
+    <col width="23.109375" customWidth="1" min="8" max="8"/>
     <col width="12.6640625" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" style="4" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="23.44140625" bestFit="1" customWidth="1" min="13" max="13"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
@@ -7310,7 +7319,11 @@
           <t>ml</t>
         </is>
       </c>
-      <c r="M103" s="2" t="n"/>
+      <c r="M103" s="2" t="inlineStr">
+        <is>
+          <t>cocktails/sangria.jpg</t>
+        </is>
+      </c>
       <c r="N103" s="2" t="b">
         <v>0</v>
       </c>
@@ -7379,7 +7392,11 @@
           <t>ml</t>
         </is>
       </c>
-      <c r="M104" s="2" t="n"/>
+      <c r="M104" s="2" t="inlineStr">
+        <is>
+          <t>cocktails/sangria.jpg</t>
+        </is>
+      </c>
       <c r="N104" s="2" t="b">
         <v>0</v>
       </c>
@@ -8542,7 +8559,7 @@
         </is>
       </c>
       <c r="J121" s="9" t="n">
-        <v>4</v>
+        <v>2.3</v>
       </c>
       <c r="K121" s="15" t="n">
         <v>330</v>
@@ -9546,7 +9563,11 @@
           <t>ml</t>
         </is>
       </c>
-      <c r="M135" s="2" t="n"/>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>cocktails/sar_tikvenik.jpg</t>
+        </is>
+      </c>
       <c r="N135" s="2" t="b">
         <v>0</v>
       </c>
@@ -10471,6 +10492,11 @@
           <t>ml</t>
         </is>
       </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>cocktails/borovinkov_oblak.jpg</t>
+        </is>
+      </c>
       <c r="N148" s="2" t="b">
         <v>0</v>
       </c>
@@ -10972,7 +10998,11 @@
           <t>g</t>
         </is>
       </c>
-      <c r="M155" s="2" t="n"/>
+      <c r="M155" s="2" t="inlineStr">
+        <is>
+          <t>food/burgers/burger_lokum.jpg</t>
+        </is>
+      </c>
       <c r="N155" s="2" t="b">
         <v>0</v>
       </c>
@@ -11045,7 +11075,11 @@
           <t>g</t>
         </is>
       </c>
-      <c r="M156" s="2" t="n"/>
+      <c r="M156" s="2" t="inlineStr">
+        <is>
+          <t>food/mains/kartoki.jpg</t>
+        </is>
+      </c>
       <c r="N156" s="2" t="b">
         <v>0</v>
       </c>
@@ -11264,7 +11298,11 @@
           <t>g</t>
         </is>
       </c>
-      <c r="M159" s="2" t="n"/>
+      <c r="M159" s="27" t="inlineStr">
+        <is>
+          <t>food/mains/rolca_narnia.jpg</t>
+        </is>
+      </c>
       <c r="N159" s="2" t="b">
         <v>0</v>
       </c>
@@ -11531,8 +11569,8 @@
       <c r="P163" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q163" t="b">
-        <v>1</v>
+      <c r="Q163" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R163" s="2" t="inlineStr">
         <is>
@@ -11602,8 +11640,8 @@
       <c r="P164" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q164" t="b">
-        <v>1</v>
+      <c r="Q164" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R164" s="2" t="inlineStr">
         <is>
@@ -11669,8 +11707,8 @@
       <c r="P165" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q165" t="b">
-        <v>1</v>
+      <c r="Q165" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R165" s="2" t="inlineStr">
         <is>
@@ -11740,8 +11778,8 @@
       <c r="P166" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q166" t="b">
-        <v>1</v>
+      <c r="Q166" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R166" s="2" t="inlineStr">
         <is>
@@ -11811,8 +11849,8 @@
       <c r="P167" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q167" t="b">
-        <v>1</v>
+      <c r="Q167" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R167" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: sort by featured/availability, light-mode contrast fix, food card redesign, drink card full-bleed image, bigger archive thumbnails
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -941,9 +941,6 @@
     <t>Heineken 330ml</t>
   </si>
   <si>
-    <t>draft</t>
-  </si>
-  <si>
     <t>limonada</t>
   </si>
   <si>
@@ -969,6 +966,9 @@
   </si>
   <si>
     <t>glarus</t>
+  </si>
+  <si>
+    <t>Наливна бира GLARUS 500ml</t>
   </si>
   <si>
     <t>Glarus 500ml</t>
@@ -1172,6 +1172,9 @@
   </si>
   <si>
     <t>dubbel</t>
+  </si>
+  <si>
+    <t>Бира Гларус Абатски Йейл</t>
   </si>
   <si>
     <t>Beer Glarus Dubbel</t>
@@ -1736,6 +1739,9 @@
     <t>nalivna_glarus</t>
   </si>
   <si>
+    <t>draft</t>
+  </si>
+  <si>
     <t>Наливна бира GLARUS 330ml</t>
   </si>
   <si>
@@ -2776,12 +2782,6 @@
   </si>
   <si>
     <t>Sulphur dioxide and sulphites (preservatives, e.g. in wine).</t>
-  </si>
-  <si>
-    <t>Бира Гларус Абатски Йейл</t>
-  </si>
-  <si>
-    <t>Наливна бира GLARUS 500ml</t>
   </si>
 </sst>
 </file>
@@ -6678,7 +6678,7 @@
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B73" t="s">
         <v>20</v>
@@ -6687,22 +6687,22 @@
         <v>65</v>
       </c>
       <c r="D73" t="s">
+        <v>308</v>
+      </c>
+      <c r="E73" t="s">
+        <v>307</v>
+      </c>
+      <c r="F73" t="s">
         <v>309</v>
       </c>
-      <c r="E73" t="s">
-        <v>308</v>
-      </c>
-      <c r="F73" t="s">
+      <c r="G73" t="s">
         <v>310</v>
       </c>
-      <c r="G73" t="s">
+      <c r="H73" t="s">
         <v>311</v>
       </c>
-      <c r="H73" t="s">
+      <c r="I73" t="s">
         <v>312</v>
-      </c>
-      <c r="I73" t="s">
-        <v>313</v>
       </c>
       <c r="J73" s="9">
         <v>3</v>
@@ -6727,12 +6727,12 @@
         <v>1</v>
       </c>
       <c r="R73" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="74" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="B74" s="2" t="s">
         <v>20</v>
@@ -6741,13 +6741,13 @@
         <v>289</v>
       </c>
       <c r="D74" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E74" t="s">
         <v>291</v>
       </c>
       <c r="F74" t="s">
-        <v>895</v>
+        <v>316</v>
       </c>
       <c r="G74" t="s">
         <v>317</v>
@@ -6762,7 +6762,7 @@
         <v>24</v>
       </c>
       <c r="N74" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O74" t="b">
         <v>0</v>
@@ -6943,7 +6943,7 @@
         <v>289</v>
       </c>
       <c r="D78" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E78" t="s">
         <v>340</v>
@@ -6970,7 +6970,7 @@
         <v>344</v>
       </c>
       <c r="N78" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O78" t="b">
         <v>0</v>
@@ -6996,7 +6996,7 @@
         <v>289</v>
       </c>
       <c r="D79" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E79" t="s">
         <v>346</v>
@@ -7023,7 +7023,7 @@
         <v>350</v>
       </c>
       <c r="N79" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O79" t="b">
         <v>0</v>
@@ -7049,7 +7049,7 @@
         <v>289</v>
       </c>
       <c r="D80" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E80" t="s">
         <v>352</v>
@@ -7076,7 +7076,7 @@
         <v>356</v>
       </c>
       <c r="N80" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O80" t="b">
         <v>0</v>
@@ -7102,7 +7102,7 @@
         <v>289</v>
       </c>
       <c r="D81" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E81" t="s">
         <v>358</v>
@@ -7126,7 +7126,7 @@
         <v>24</v>
       </c>
       <c r="N81" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O81" t="b">
         <v>0</v>
@@ -7152,7 +7152,7 @@
         <v>289</v>
       </c>
       <c r="D82" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E82" t="s">
         <v>363</v>
@@ -7176,7 +7176,7 @@
         <v>24</v>
       </c>
       <c r="N82" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O82" t="b">
         <v>0</v>
@@ -7202,19 +7202,19 @@
         <v>289</v>
       </c>
       <c r="D83" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E83" t="s">
         <v>368</v>
       </c>
       <c r="F83" t="s">
-        <v>894</v>
+        <v>369</v>
       </c>
       <c r="G83" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="H83" s="26" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="J83" s="9">
         <v>3.3</v>
@@ -7226,7 +7226,7 @@
         <v>24</v>
       </c>
       <c r="N83" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O83" t="b">
         <v>0</v>
@@ -7243,7 +7243,7 @@
     </row>
     <row r="84" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B84" t="s">
         <v>20</v>
@@ -7252,19 +7252,19 @@
         <v>289</v>
       </c>
       <c r="D84" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="E84" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F84" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G84" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="H84" s="26" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J84" s="9">
         <v>3.3</v>
@@ -7276,7 +7276,7 @@
         <v>24</v>
       </c>
       <c r="N84" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O84" t="b">
         <v>0</v>
@@ -7293,7 +7293,7 @@
     </row>
     <row r="85" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B85" s="2" t="s">
         <v>20</v>
@@ -7302,16 +7302,16 @@
         <v>70</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H85" s="2"/>
       <c r="I85" s="2"/>
@@ -7344,7 +7344,7 @@
     </row>
     <row r="86" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B86" s="2" t="s">
         <v>47</v>
@@ -7355,10 +7355,10 @@
       <c r="D86" s="2"/>
       <c r="E86" s="2"/>
       <c r="F86" s="2" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="H86" s="2"/>
       <c r="I86" s="2"/>
@@ -7391,7 +7391,7 @@
     </row>
     <row r="87" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B87" s="2" t="s">
         <v>47</v>
@@ -7402,10 +7402,10 @@
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
       <c r="F87" s="2" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="H87" s="2"/>
       <c r="I87" s="2"/>
@@ -7438,7 +7438,7 @@
     </row>
     <row r="88" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B88" s="2" t="s">
         <v>47</v>
@@ -7449,10 +7449,10 @@
       <c r="D88" s="2"/>
       <c r="E88" s="2"/>
       <c r="F88" s="2" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="H88" s="2"/>
       <c r="I88" s="2"/>
@@ -7485,7 +7485,7 @@
     </row>
     <row r="89" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B89" s="2" t="s">
         <v>47</v>
@@ -7496,16 +7496,16 @@
       <c r="D89" s="2"/>
       <c r="E89" s="2"/>
       <c r="F89" s="2" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="H89" s="2" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="I89" s="2" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="J89" s="8">
         <v>3.5</v>
@@ -7533,12 +7533,12 @@
         <v>62</v>
       </c>
       <c r="S89" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="90" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B90" s="2" t="s">
         <v>47</v>
@@ -7549,10 +7549,10 @@
       <c r="D90" s="2"/>
       <c r="E90" s="2"/>
       <c r="F90" s="2" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="H90" s="2"/>
       <c r="I90" s="2"/>
@@ -7585,7 +7585,7 @@
     </row>
     <row r="91" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B91" s="2" t="s">
         <v>20</v>
@@ -7594,16 +7594,16 @@
         <v>70</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F91" s="2" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="H91" s="2"/>
       <c r="I91" s="2"/>
@@ -7630,33 +7630,33 @@
         <v>1</v>
       </c>
       <c r="R91" s="2" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="S91" s="2"/>
     </row>
     <row r="92" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
       <c r="F92" s="2" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H92" s="2" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="I92" s="2" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="J92" s="8">
         <v>3.6</v>
@@ -7681,7 +7681,7 @@
         <v>1</v>
       </c>
       <c r="R92" s="2" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="S92" s="2" t="s">
         <v>63</v>
@@ -7689,27 +7689,27 @@
     </row>
     <row r="93" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B93" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D93" s="2"/>
       <c r="E93" s="2"/>
       <c r="F93" s="2" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="H93" s="2" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="I93" s="2" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="J93" s="8">
         <v>3.6</v>
@@ -7734,33 +7734,33 @@
         <v>1</v>
       </c>
       <c r="R93" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S93" s="2"/>
     </row>
     <row r="94" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B94" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
       <c r="F94" s="2" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="I94" s="2" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="J94" s="8">
         <v>3.6</v>
@@ -7785,35 +7785,35 @@
         <v>1</v>
       </c>
       <c r="R94" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S94" s="2" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="95" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B95" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
       <c r="F95" s="2" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="H95" s="2" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="I95" s="2" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="J95" s="8">
         <v>3.6</v>
@@ -7838,33 +7838,33 @@
         <v>1</v>
       </c>
       <c r="R95" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S95" s="2"/>
     </row>
     <row r="96" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B96" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D96" s="2"/>
       <c r="E96" s="2"/>
       <c r="F96" s="2" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="I96" s="2" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J96" s="8">
         <v>3.6</v>
@@ -7889,33 +7889,33 @@
         <v>1</v>
       </c>
       <c r="R96" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S96" s="2"/>
     </row>
     <row r="97" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="B97" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
       <c r="F97" s="2" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="I97" s="2" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="J97" s="8">
         <v>3.6</v>
@@ -7940,33 +7940,33 @@
         <v>1</v>
       </c>
       <c r="R97" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S97" s="2"/>
     </row>
     <row r="98" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="B98" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
       <c r="F98" s="2" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H98" s="2" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="I98" s="2" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="J98" s="8">
         <v>3.6</v>
@@ -7991,33 +7991,33 @@
         <v>1</v>
       </c>
       <c r="R98" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S98" s="2"/>
     </row>
     <row r="99" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="B99" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D99" s="2"/>
       <c r="E99" s="2"/>
       <c r="F99" s="2" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I99" s="2" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J99" s="8">
         <v>3.6</v>
@@ -8042,33 +8042,33 @@
         <v>1</v>
       </c>
       <c r="R99" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S99" s="2"/>
     </row>
     <row r="100" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B100" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D100" s="2"/>
       <c r="E100" s="2"/>
       <c r="F100" s="2" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="H100" s="2" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="I100" s="2" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="J100" s="8">
         <v>3.6</v>
@@ -8093,33 +8093,33 @@
         <v>1</v>
       </c>
       <c r="R100" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S100" s="2"/>
     </row>
     <row r="101" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B101" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D101" s="2"/>
       <c r="E101" s="2"/>
       <c r="F101" s="2" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="H101" s="2" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I101" s="2" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J101" s="8">
         <v>3.6</v>
@@ -8144,33 +8144,33 @@
         <v>1</v>
       </c>
       <c r="R101" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S101" s="2"/>
     </row>
     <row r="102" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="B102" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
       <c r="F102" s="2" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="H102" s="2" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="I102" s="2" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J102" s="8">
         <v>3.6</v>
@@ -8182,7 +8182,7 @@
         <v>24</v>
       </c>
       <c r="M102" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N102" s="2" t="b">
         <v>0</v>
@@ -8197,33 +8197,33 @@
         <v>1</v>
       </c>
       <c r="R102" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S102" s="2"/>
     </row>
     <row r="103" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
       <c r="F103" s="2" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="I103" s="2" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J103" s="8">
         <v>3.6</v>
@@ -8235,7 +8235,7 @@
         <v>24</v>
       </c>
       <c r="M103" s="2" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="N103" s="2" t="b">
         <v>0</v>
@@ -8250,13 +8250,13 @@
         <v>1</v>
       </c>
       <c r="R103" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S103" s="2"/>
     </row>
     <row r="104" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B104" s="2" t="s">
         <v>47</v>
@@ -8267,16 +8267,16 @@
       <c r="D104" s="2"/>
       <c r="E104" s="2"/>
       <c r="F104" s="2" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="H104" s="2" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="I104" s="2" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="J104" s="8">
         <v>3.8</v>
@@ -8304,12 +8304,12 @@
         <v>324</v>
       </c>
       <c r="S104" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="105" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="B105" s="2" t="s">
         <v>47</v>
@@ -8320,10 +8320,10 @@
       <c r="D105" s="2"/>
       <c r="E105" s="2"/>
       <c r="F105" s="2" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="H105" s="2"/>
       <c r="I105" s="2"/>
@@ -8356,7 +8356,7 @@
     </row>
     <row r="106" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>47</v>
@@ -8367,16 +8367,16 @@
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
       <c r="F106" s="2" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="H106" s="2" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="I106" s="2" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="J106" s="8">
         <v>3.8</v>
@@ -8404,32 +8404,32 @@
         <v>62</v>
       </c>
       <c r="S106" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="107" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D107" s="2"/>
       <c r="E107" s="2"/>
       <c r="F107" s="2" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="H107" s="2" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="I107" s="2" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J107" s="10">
         <v>3.8</v>
@@ -8454,13 +8454,13 @@
         <v>1</v>
       </c>
       <c r="R107" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S107" s="2"/>
     </row>
     <row r="108" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>47</v>
@@ -8471,16 +8471,16 @@
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
       <c r="F108" s="2" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="H108" s="2" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="I108" s="2" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J108" s="10">
         <v>3.9</v>
@@ -8508,12 +8508,12 @@
         <v>62</v>
       </c>
       <c r="S108" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="109" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>47</v>
@@ -8524,10 +8524,10 @@
       <c r="D109" s="2"/>
       <c r="E109" s="2"/>
       <c r="F109" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="H109" s="2"/>
       <c r="I109" s="2"/>
@@ -8560,27 +8560,27 @@
     </row>
     <row r="110" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D110" s="2"/>
       <c r="E110" s="2"/>
       <c r="F110" s="2" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I110" s="2" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="J110" s="8">
         <v>4</v>
@@ -8605,33 +8605,33 @@
         <v>1</v>
       </c>
       <c r="R110" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S110" s="2"/>
     </row>
     <row r="111" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D111" s="2"/>
       <c r="E111" s="2"/>
       <c r="F111" s="2" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="I111" s="2" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J111" s="8">
         <v>4</v>
@@ -8656,33 +8656,33 @@
         <v>1</v>
       </c>
       <c r="R111" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S111" s="2"/>
     </row>
     <row r="112" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
       <c r="F112" s="2" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="H112" s="2" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="I112" s="2" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J112" s="8">
         <v>4</v>
@@ -8707,33 +8707,33 @@
         <v>1</v>
       </c>
       <c r="R112" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S112" s="2"/>
     </row>
     <row r="113" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D113" s="2"/>
       <c r="E113" s="2"/>
       <c r="F113" s="2" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="H113" s="2" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="I113" s="2" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="J113" s="8">
         <v>4</v>
@@ -8758,33 +8758,33 @@
         <v>1</v>
       </c>
       <c r="R113" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S113" s="2"/>
     </row>
     <row r="114" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
       <c r="F114" s="2" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="H114" s="2" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="I114" s="2" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J114" s="8">
         <v>4</v>
@@ -8809,33 +8809,33 @@
         <v>1</v>
       </c>
       <c r="R114" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S114" s="2"/>
     </row>
     <row r="115" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D115" s="2"/>
       <c r="E115" s="2"/>
       <c r="F115" s="2" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="H115" s="2" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="I115" s="2" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="J115" s="8">
         <v>4</v>
@@ -8860,33 +8860,33 @@
         <v>1</v>
       </c>
       <c r="R115" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S115" s="2"/>
     </row>
     <row r="116" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
       <c r="F116" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="H116" s="2" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="I116" s="2" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J116" s="8">
         <v>4</v>
@@ -8911,33 +8911,33 @@
         <v>1</v>
       </c>
       <c r="R116" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S116" s="2"/>
     </row>
     <row r="117" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D117" s="2"/>
       <c r="E117" s="2"/>
       <c r="F117" s="2" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="H117" s="2" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="I117" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="J117" s="8">
         <v>4</v>
@@ -8962,33 +8962,33 @@
         <v>1</v>
       </c>
       <c r="R117" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S117" s="2"/>
     </row>
     <row r="118" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B118" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
       <c r="F118" s="2" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="H118" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="I118" s="2" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J118" s="8">
         <v>4</v>
@@ -9013,7 +9013,7 @@
         <v>1</v>
       </c>
       <c r="R118" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S118" s="2" t="s">
         <v>63</v>
@@ -9021,27 +9021,27 @@
     </row>
     <row r="119" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
       <c r="F119" s="2" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="H119" s="2" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="I119" s="2" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="J119" s="8">
         <v>4</v>
@@ -9064,7 +9064,7 @@
         <v>1</v>
       </c>
       <c r="R119" s="2" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="S119" s="2" t="s">
         <v>63</v>
@@ -9072,7 +9072,7 @@
     </row>
     <row r="120" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B120" t="s">
         <v>20</v>
@@ -9081,16 +9081,16 @@
         <v>289</v>
       </c>
       <c r="D120" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E120" t="s">
-        <v>307</v>
+        <v>548</v>
       </c>
       <c r="F120" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="G120" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="J120" s="9">
         <v>2.2999999999999998</v>
@@ -9102,7 +9102,7 @@
         <v>24</v>
       </c>
       <c r="N120" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O120" t="b">
         <v>0</v>
@@ -9114,30 +9114,30 @@
         <v>1</v>
       </c>
       <c r="R120" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="121" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B121" t="s">
         <v>20</v>
       </c>
       <c r="C121" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D121" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E121" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F121" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G121" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="J121" s="9">
         <v>4</v>
@@ -9161,30 +9161,30 @@
         <v>1</v>
       </c>
       <c r="R121" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="122" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="B122" t="s">
         <v>20</v>
       </c>
       <c r="C122" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D122" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E122" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F122" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="G122" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="J122" s="9">
         <v>4</v>
@@ -9208,30 +9208,30 @@
         <v>1</v>
       </c>
       <c r="R122" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="123" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="B123" t="s">
         <v>20</v>
       </c>
       <c r="C123" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D123" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E123" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F123" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="G123" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="J123" s="9">
         <v>4</v>
@@ -9255,36 +9255,36 @@
         <v>1</v>
       </c>
       <c r="R123" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="124" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C124" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D124" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E124" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="F124" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="G124" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="H124" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="I124" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="J124" s="9">
         <v>4</v>
@@ -9308,36 +9308,36 @@
         <v>1</v>
       </c>
       <c r="R124" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="125" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C125" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D125" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E125" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F125" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="G125" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="H125" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="I125" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="J125" s="9">
         <v>4</v>
@@ -9361,36 +9361,36 @@
         <v>1</v>
       </c>
       <c r="R125" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="126" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C126" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D126" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E126" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F126" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G126" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="H126" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="I126" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="J126" s="9">
         <v>4</v>
@@ -9414,36 +9414,36 @@
         <v>1</v>
       </c>
       <c r="R126" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="127" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C127" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D127" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E127" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F127" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G127" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="H127" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="I127" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="J127" s="9">
         <v>4</v>
@@ -9467,36 +9467,36 @@
         <v>1</v>
       </c>
       <c r="R127" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="128" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C128" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D128" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E128" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="F128" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="G128" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="H128" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="I128" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="J128" s="9">
         <v>4</v>
@@ -9520,36 +9520,36 @@
         <v>1</v>
       </c>
       <c r="R128" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="129" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C129" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D129" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E129" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F129" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="G129" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="H129" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="I129" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="J129" s="9">
         <v>4</v>
@@ -9573,36 +9573,36 @@
         <v>1</v>
       </c>
       <c r="R129" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="130" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C130" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D130" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E130" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="F130" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="G130" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="H130" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="I130" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="J130" s="9">
         <v>4</v>
@@ -9626,12 +9626,12 @@
         <v>1</v>
       </c>
       <c r="R130" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="131" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>47</v>
@@ -9642,10 +9642,10 @@
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
       <c r="F131" s="2" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="H131" s="2"/>
       <c r="I131" s="2"/>
@@ -9678,7 +9678,7 @@
     </row>
     <row r="132" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>47</v>
@@ -9689,16 +9689,16 @@
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
       <c r="F132" s="2" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="I132" s="2" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="J132" s="18">
         <v>4.0999999999999996</v>
@@ -9731,7 +9731,7 @@
     </row>
     <row r="133" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>47</v>
@@ -9742,16 +9742,16 @@
       <c r="D133" s="2"/>
       <c r="E133" s="2"/>
       <c r="F133" s="2" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="G133" s="2" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="I133" s="2" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="J133" s="8">
         <v>4.0999999999999996</v>
@@ -9779,32 +9779,32 @@
         <v>62</v>
       </c>
       <c r="S133" s="2" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
     </row>
     <row r="134" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D134" s="2"/>
       <c r="E134" s="2"/>
       <c r="F134" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="H134" s="2" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="I134" s="2" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="J134" s="8">
         <v>4.0999999999999996</v>
@@ -9816,7 +9816,7 @@
         <v>24</v>
       </c>
       <c r="M134" s="2" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="N134" s="2" t="b">
         <v>0</v>
@@ -9831,13 +9831,13 @@
         <v>1</v>
       </c>
       <c r="R134" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="S134" s="2"/>
     </row>
     <row r="135" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>20</v>
@@ -9846,16 +9846,16 @@
         <v>70</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>71</v>
       </c>
       <c r="F135" s="2" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="H135" s="2"/>
       <c r="I135" s="2"/>
@@ -9888,7 +9888,7 @@
     </row>
     <row r="136" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>327</v>
@@ -9899,16 +9899,16 @@
       <c r="D136" s="2"/>
       <c r="E136" s="2"/>
       <c r="F136" s="2" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="H136" s="2" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="I136" s="2" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="J136" s="8">
         <v>4.3499999999999996</v>
@@ -9933,13 +9933,13 @@
         <v>1</v>
       </c>
       <c r="R136" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="S136" s="2"/>
     </row>
     <row r="137" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B137" s="2" t="s">
         <v>327</v>
@@ -9950,16 +9950,16 @@
       <c r="D137" s="2"/>
       <c r="E137" s="2"/>
       <c r="F137" s="2" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="G137" s="2" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="I137" s="2" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="J137" s="8">
         <v>4.3499999999999996</v>
@@ -9984,13 +9984,13 @@
         <v>1</v>
       </c>
       <c r="R137" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="S137" s="2"/>
     </row>
     <row r="138" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>327</v>
@@ -10001,16 +10001,16 @@
       <c r="D138" s="2"/>
       <c r="E138" s="2"/>
       <c r="F138" s="2" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="G138" s="2" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="I138" s="2" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="J138" s="8">
         <v>4.4000000000000004</v>
@@ -10035,13 +10035,13 @@
         <v>1</v>
       </c>
       <c r="R138" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="S138" s="2"/>
     </row>
     <row r="139" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>327</v>
@@ -10052,16 +10052,16 @@
       <c r="D139" s="2"/>
       <c r="E139" s="2"/>
       <c r="F139" s="2" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="G139" s="2" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="H139" s="2" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="I139" s="2" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="J139" s="8">
         <v>4.4000000000000004</v>
@@ -10086,33 +10086,33 @@
         <v>1</v>
       </c>
       <c r="R139" s="2" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="S139" s="2"/>
     </row>
     <row r="140" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C140" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D140" s="2"/>
       <c r="E140" s="2"/>
       <c r="F140" s="2" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="G140" s="2" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="I140" s="2" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="J140" s="8">
         <v>4.4000000000000004</v>
@@ -10137,15 +10137,15 @@
         <v>1</v>
       </c>
       <c r="R140" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S140" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="141" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>20</v>
@@ -10154,16 +10154,16 @@
         <v>70</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>96</v>
       </c>
       <c r="F141" s="2" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="G141" s="2" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="H141" s="2"/>
       <c r="I141" s="2"/>
@@ -10196,7 +10196,7 @@
     </row>
     <row r="142" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>47</v>
@@ -10207,16 +10207,16 @@
       <c r="D142" s="2"/>
       <c r="E142" s="2"/>
       <c r="F142" s="2" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G142" s="2" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="I142" s="2" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="J142" s="8">
         <v>4.5999999999999996</v>
@@ -10244,12 +10244,12 @@
         <v>324</v>
       </c>
       <c r="S142" s="2" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="143" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>47</v>
@@ -10260,10 +10260,10 @@
       <c r="D143" s="2"/>
       <c r="E143" s="2"/>
       <c r="F143" s="2" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="G143" s="2" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="H143" s="2"/>
       <c r="I143" s="2"/>
@@ -10293,32 +10293,32 @@
         <v>324</v>
       </c>
       <c r="S143" s="2" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="144" spans="1:19" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C144" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D144" s="2"/>
       <c r="E144" s="2"/>
       <c r="F144" s="2" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="G144" s="2" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="I144" s="2" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="J144" s="8">
         <v>4.9000000000000004</v>
@@ -10343,39 +10343,39 @@
         <v>1</v>
       </c>
       <c r="R144" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S144" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="145" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C145" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D145" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E145" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="F145" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="G145" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="H145" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="I145" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="J145" s="9">
         <v>5</v>
@@ -10399,36 +10399,36 @@
         <v>1</v>
       </c>
       <c r="R145" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="146" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C146" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D146" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E146" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F146" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="G146" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="H146" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="I146" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="J146" s="9">
         <v>5</v>
@@ -10452,36 +10452,36 @@
         <v>1</v>
       </c>
       <c r="R146" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="147" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="B147" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C147" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D147" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E147" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="F147" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="G147" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="H147" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="I147" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="J147" s="9">
         <v>5</v>
@@ -10493,7 +10493,7 @@
         <v>24</v>
       </c>
       <c r="M147" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="N147" s="2" t="b">
         <v>0</v>
@@ -10508,36 +10508,36 @@
         <v>1</v>
       </c>
       <c r="R147" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="148" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C148" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D148" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E148" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F148" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="G148" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="H148" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="I148" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="J148" s="9">
         <v>5</v>
@@ -10561,36 +10561,36 @@
         <v>1</v>
       </c>
       <c r="R148" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="149" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>327</v>
       </c>
       <c r="C149" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D149" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="E149" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="F149" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="G149" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="H149" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="I149" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="J149" s="9">
         <v>5</v>
@@ -10614,12 +10614,12 @@
         <v>1</v>
       </c>
       <c r="R149" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
     </row>
     <row r="150" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>47</v>
@@ -10630,10 +10630,10 @@
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
       <c r="F150" s="2" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="G150" s="2" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="H150" s="2"/>
       <c r="I150" s="2"/>
@@ -10663,12 +10663,12 @@
         <v>324</v>
       </c>
       <c r="S150" s="2" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="151" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>47</v>
@@ -10679,16 +10679,16 @@
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
       <c r="F151" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="G151" s="2" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="I151" s="2" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="J151" s="8">
         <v>5.6</v>
@@ -10716,12 +10716,12 @@
         <v>324</v>
       </c>
       <c r="S151" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="152" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>47</v>
@@ -10732,16 +10732,16 @@
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
       <c r="F152" s="2" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="G152" s="2" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="I152" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="J152" s="8">
         <v>6</v>
@@ -10769,32 +10769,32 @@
         <v>324</v>
       </c>
       <c r="S152" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="153" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="D153" s="2"/>
       <c r="E153" s="2"/>
       <c r="F153" s="2" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="I153" s="2" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="J153" s="18">
         <v>6</v>
@@ -10819,35 +10819,35 @@
         <v>1</v>
       </c>
       <c r="R153" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="S153" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="154" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D154" s="2"/>
       <c r="E154" s="2"/>
       <c r="F154" s="2" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="I154" s="2" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="J154" s="8">
         <v>6.4</v>
@@ -10859,7 +10859,7 @@
         <v>61</v>
       </c>
       <c r="M154" s="2" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="N154" s="2" t="b">
         <v>0</v>
@@ -10874,15 +10874,15 @@
         <v>1</v>
       </c>
       <c r="R154" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S154" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="155" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>47</v>
@@ -10893,16 +10893,16 @@
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
       <c r="F155" s="2" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="H155" s="2" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="I155" s="2" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="J155" s="8">
         <v>6.5</v>
@@ -10914,7 +10914,7 @@
         <v>61</v>
       </c>
       <c r="M155" s="2" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="N155" s="2" t="b">
         <v>0</v>
@@ -10937,27 +10937,27 @@
     </row>
     <row r="156" spans="1:19" ht="138" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
       <c r="F156" s="2" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="H156" s="2" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="J156" s="18">
         <v>7.5</v>
@@ -10982,15 +10982,15 @@
         <v>1</v>
       </c>
       <c r="R156" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="S156" s="2" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
     </row>
     <row r="157" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>47</v>
@@ -11001,16 +11001,16 @@
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
       <c r="F157" s="2" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="I157" s="2" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="J157" s="8">
         <v>7.9</v>
@@ -11038,12 +11038,12 @@
         <v>324</v>
       </c>
       <c r="S157" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="158" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>47</v>
@@ -11054,16 +11054,16 @@
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
       <c r="F158" s="2" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="H158" s="2" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="I158" s="2" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="J158" s="8">
         <v>9.5</v>
@@ -11075,7 +11075,7 @@
         <v>61</v>
       </c>
       <c r="M158" s="27" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="N158" s="2" t="b">
         <v>0</v>
@@ -11098,25 +11098,25 @@
     </row>
     <row r="159" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B159" t="s">
         <v>20</v>
       </c>
       <c r="C159" s="21" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D159" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E159" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F159" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="G159" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="J159" s="9">
         <v>12</v>
@@ -11142,25 +11142,25 @@
     </row>
     <row r="160" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="B160" t="s">
         <v>20</v>
       </c>
       <c r="C160" s="21" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D160" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E160" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F160" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="G160" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="J160" s="9">
         <v>12</v>
@@ -11186,25 +11186,25 @@
     </row>
     <row r="161" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="B161" t="s">
         <v>20</v>
       </c>
       <c r="C161" s="21" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D161" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E161" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F161" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="G161" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="J161" s="9">
         <v>12</v>
@@ -11230,7 +11230,7 @@
     </row>
     <row r="162" spans="1:19" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>47</v>
@@ -11241,16 +11241,16 @@
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
       <c r="F162" s="12" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="G162" s="12" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="H162" s="12" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="I162" s="12" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="J162" s="22"/>
       <c r="K162" s="16">
@@ -11276,12 +11276,12 @@
         <v>324</v>
       </c>
       <c r="S162" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="163" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>20</v>
@@ -11290,16 +11290,16 @@
         <v>70</v>
       </c>
       <c r="D163" s="2" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="F163" s="12" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="G163" s="12" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="H163" s="12"/>
       <c r="I163" s="12"/>
@@ -11330,27 +11330,27 @@
     </row>
     <row r="164" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D164" s="2"/>
       <c r="E164" s="2"/>
       <c r="F164" s="12" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="G164" s="12" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="H164" s="12" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="I164" s="12" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="J164" s="22"/>
       <c r="K164" s="16">
@@ -11373,35 +11373,35 @@
         <v>0</v>
       </c>
       <c r="R164" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S164" s="2" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
     </row>
     <row r="165" spans="1:19" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D165" s="2"/>
       <c r="E165" s="2"/>
       <c r="F165" s="12" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="G165" s="12" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="H165" s="12" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="I165" s="12" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="J165" s="22"/>
       <c r="K165" s="16">
@@ -11424,35 +11424,35 @@
         <v>0</v>
       </c>
       <c r="R165" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S165" s="2" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
     </row>
     <row r="166" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
       <c r="F166" s="12" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="G166" s="12" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="H166" s="12" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="I166" s="12" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="J166" s="22"/>
       <c r="K166" s="16">
@@ -11475,35 +11475,35 @@
         <v>0</v>
       </c>
       <c r="R166" s="2" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="S166" s="2" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
     </row>
     <row r="167" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D167" s="2"/>
       <c r="E167" s="2"/>
       <c r="F167" s="12" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="G167" s="12" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="H167" s="12" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="I167" s="12" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="J167" s="22">
         <v>3.3</v>
@@ -11515,7 +11515,7 @@
         <v>61</v>
       </c>
       <c r="M167" s="2" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="N167" s="2" t="b">
         <v>0</v>
@@ -11530,35 +11530,35 @@
         <v>1</v>
       </c>
       <c r="R167" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S167" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="168" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
       <c r="F168" s="12" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="G168" s="12" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="H168" s="12" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="I168" s="12" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="J168" s="22">
         <v>6.9</v>
@@ -11583,35 +11583,35 @@
         <v>1</v>
       </c>
       <c r="R168" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S168" s="2" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
     </row>
     <row r="169" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
       <c r="F169" s="12" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="G169" s="12" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="H169" s="12" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="I169" s="12" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="J169" s="22">
         <v>3.4</v>
@@ -11636,35 +11636,35 @@
         <v>1</v>
       </c>
       <c r="R169" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S169" s="2" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="170" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C170" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
       <c r="F170" s="12" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="G170" s="12" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="H170" s="12" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="I170" s="12" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="J170" s="22">
         <v>3.1</v>
@@ -11676,7 +11676,7 @@
         <v>61</v>
       </c>
       <c r="M170" s="2" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="N170" s="2" t="b">
         <v>0</v>
@@ -11691,7 +11691,7 @@
         <v>1</v>
       </c>
       <c r="R170" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S170" s="25" t="s">
         <v>325</v>
@@ -11699,27 +11699,27 @@
     </row>
     <row r="171" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D171" s="2"/>
       <c r="E171" s="2"/>
       <c r="F171" s="12" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="G171" s="12" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="H171" s="12" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="I171" s="12" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="J171" s="22">
         <v>4.9000000000000004</v>
@@ -11744,29 +11744,29 @@
         <v>1</v>
       </c>
       <c r="R171" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S171" s="25" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
     </row>
     <row r="172" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="D172" s="2"/>
       <c r="E172" s="2"/>
       <c r="F172" s="12" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="G172" s="12" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="H172" s="12"/>
       <c r="I172" s="12"/>
@@ -11791,15 +11791,15 @@
         <v>1</v>
       </c>
       <c r="R172" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="S172" s="25" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
     </row>
     <row r="173" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>327</v>
@@ -11810,16 +11810,16 @@
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
       <c r="F173" s="12" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="G173" s="12" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="H173" s="12" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="I173" s="12" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
       <c r="J173" s="22">
         <v>3.3</v>
@@ -11844,13 +11844,13 @@
         <v>1</v>
       </c>
       <c r="R173" s="2" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="S173" s="2"/>
     </row>
     <row r="174" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="B174" t="s">
         <v>20</v>
@@ -11859,10 +11859,10 @@
         <v>21</v>
       </c>
       <c r="F174" s="13" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="G174" s="13" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="H174" s="13"/>
       <c r="I174" s="13"/>
@@ -11891,7 +11891,7 @@
     </row>
     <row r="175" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="B175" t="s">
         <v>20</v>
@@ -11900,10 +11900,10 @@
         <v>30</v>
       </c>
       <c r="F175" s="13" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="G175" s="13" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="H175" s="13"/>
       <c r="I175" s="13"/>
@@ -11932,7 +11932,7 @@
     </row>
     <row r="176" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="B176" t="s">
         <v>20</v>
@@ -11941,10 +11941,10 @@
         <v>30</v>
       </c>
       <c r="F176" s="14" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="G176" s="13" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="H176" s="13"/>
       <c r="I176" s="13"/>
@@ -11970,7 +11970,7 @@
     </row>
     <row r="177" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B177" t="s">
         <v>20</v>
@@ -12016,7 +12016,7 @@
     </row>
     <row r="178" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="B178" t="s">
         <v>20</v>
@@ -12025,10 +12025,10 @@
         <v>65</v>
       </c>
       <c r="F178" s="13" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="G178" s="13" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="H178" s="13"/>
       <c r="I178" s="13"/>
@@ -12078,16 +12078,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="C1" s="24" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
       <c r="D1" s="24" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -12095,16 +12095,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="C2" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="D2" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
       <c r="E2" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -12112,16 +12112,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="C3" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
       <c r="D3" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
       <c r="E3" t="s">
-        <v>847</v>
+        <v>849</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -12129,16 +12129,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="C4" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="D4" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
       <c r="E4" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -12146,16 +12146,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="C5" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="D5" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="E5" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -12169,10 +12169,10 @@
         <v>271</v>
       </c>
       <c r="D6" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="E6" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -12180,16 +12180,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="C7" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="D7" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
       <c r="E7" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -12197,16 +12197,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="C8" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="D8" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="E8" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -12214,16 +12214,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="C9" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="D9" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="E9" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -12231,16 +12231,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
       <c r="C10" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="D10" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="E10" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -12248,16 +12248,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="C11" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
       <c r="D11" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="E11" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -12265,16 +12265,16 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="C12" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="D12" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
       <c r="E12" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -12282,16 +12282,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C13" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="D13" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="E13" t="s">
-        <v>885</v>
+        <v>887</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -12299,16 +12299,16 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="C14" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="D14" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="E14" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -12316,16 +12316,16 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
       <c r="C15" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="D15" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="E15" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: bundle Nunito/Unbounded fonts locally instead of google_fonts runtime fetch
Blank white screen on poor/no connectivity was caused by google_fonts
fetching font files from Google's CDN at runtime - if that fetch fails
(no internet, only local network), it throws uncaught and the whole app
fails to render. Fonts are now bundled as local assets, no network needed.

Also: spelling fixes in products_master.xlsx, dead tools/ scripts removed,
new archive event photos.
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -3739,7 +3739,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>РАКИЯ ТРОЯНСКА СЛИВОВА ОТЛЕЖАЛA</t>
+          <t>РАКИЯ ТРОЯНСКА СЛИВОВА ОТЛЕЖАЛА</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>Светла бира направена по технологията на "ейла". Популярна във Великобритания и САЩ сред любителите на крафт бира, заради многобройните възможни комбинации от хмел и малц, които водят до много интересни резултати. В нашия вариант сме използвали aмерикански и словенски хмел, които се допълват отлично и придават свежо усещане на цитрус. Ще задоволим всяка жажда.
+          <t>Светла бира направена по технологията на "ейла". Популярна във Великобритания и САЩ сред любителите на крафт бира, заради многобройните възможни комбинации от хмел и малц, които водят до много интересни резултати. В нашия вариант сме използвали американски и словенски хмел, които се допълват отлично и придават свежо усещане на цитрус. Ще задоволим всяка жажда.
 Стил: Pale Ale
 Алкохолен градус: 4.2%
 Съставки: вода, 3 вида светъл и ароматен малц, 2 вида хмел, бирена мая 
@@ -5594,9 +5594,9 @@
       </c>
       <c r="H79" s="26" t="inlineStr">
         <is>
-          <t>Special English Ale - най-популярната и обичана бира в Англия. Истинска класика! Mоже би най-разпространеният вид бира във Великобритания.
-Стилово нашият "Специален Ейл" съответства на англииския вариант "best/premium/special ale". Наименованието се дължи на количеството и качеството на суровините, както и на алкохолното съдържание, което е малко по-високо в сравнение с обикновения ейл "ordinary bitter". Пред вас е една изключително приятна пивка бира, на която може да се насладите по всяко време.
-Стил: Special/Best/Premium English Bitter Алкохолен
+          <t>Special English Ale - най-популярната и обичана бира в Англия. Истинска класика! Може би най-разпространеният вид бира във Великобритания.
+Стилово нашият "Специален Ейл" съответства на английския вариант "best/premium/special ale". Наименованието се дължи на количеството и качеството на суровините, както и на алкохолното съдържание, което е малко по-високо в сравнение с обикновения ейл "ordinary bitter". Пред вас е една изключително приятна пивка бира, на която може да се насладите по всяко време.
+Стил: Special/Best/Premium English Bitter
 Алкохолен градус: 4.6% 
 Съставки: вода, карамелен и светъл малц, 2 вида хмел, бирена мая 
 Цвят: тъмно златист/ кехлибарен
@@ -5766,7 +5766,7 @@
       </c>
       <c r="H81" s="26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Базирана е на на стила "Saison" (буквално "сезонна" бира), който е популярен не само в Белгия, но и сред крафт пивоварите по света. Ние също сме фенове, защото този стил позволява доста "творческа свобода" по отношение на възможните комбинации на малц, хмел и подправки. Въпреки това има едно основно правило, които ние също спазваме - бирата да е със сравнително сух завършек, което е резултат от използването на оригиналната белгийска мая и специфичната технология на ферментация.
+          <t xml:space="preserve">Базирана е на стила "Saison" (буквално "сезонна" бира), който е популярен не само в Белгия, но и сред крафт пивоварите по света. Ние също сме фенове, защото този стил позволява доста "творческа свобода" по отношение на възможните комбинации на малц, хмел и подправки. Въпреки това има едно основно правило, които ние също спазваме - бирата да е със сравнително сух завършек, което е резултат от използването на оригиналната белгийска мая и специфичната технология на ферментация.
 "SAISON на Гларус е идеалната бира за лятото - плодовите нотки и леко пиперливият вкус ще ви ободрят и освежат, а сухият завършек ще спомогне да намали жаждата ви.
 Стил: Saison
 Алкохолен градус: 5% 
@@ -5938,7 +5938,7 @@
 Лимитирана серия с богат малцов профил, мек вкус и отлична пивкост.
 Отличава се с дълбок тъмнокехлибарен до кафяв цвят, аромат на карамел, тъмен малц и сушени плодове, и балансиран, леко сладък вкус с топъл финал.
 Стил: Dubbel
-Алкохолен градус: 6.5% .
+Алкохолен градус: 6.5%.
 Състав: малц, хмел, мусковадо, белгийска бирена мая, вода
 Цвят: тъмен кехлибар до кафяв, с кремообразна пяна
 Аромат: карамел, тъмен малц, сушени плодове, леки пикантни нотки
@@ -11910,7 +11910,7 @@
       </c>
       <c r="H168" s="12" t="inlineStr">
         <is>
-          <t>Пухкаво хлебче, авокадо,пушена сьомга,домат,яйце и салата микс</t>
+          <t>Пухкаво хлебче, авокадо, пушена сьомга, домат, яйце и салата микс</t>
         </is>
       </c>
       <c r="I168" s="12" t="inlineStr">
@@ -11983,13 +11983,12 @@
       </c>
       <c r="H169" s="12" t="inlineStr">
         <is>
-          <t>С гарнитура по избор - сирене,мед,сладко от боровинки /пълнозърнест хляб, яйце, мляко и брашно</t>
+          <t>С гарнитура по избор - сирене, мед, сладко от боровинки /пълнозърнест хляб, яйце, мляко и брашно</t>
         </is>
       </c>
       <c r="I169" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-Served with a choice of accompaniment – ​​cheese, honey, or blueberry jam; includes whole-grain bread, egg, milk, and flour</t>
+          <t>Served with a choice of accompaniment – cheese, honey, or blueberry jam; includes whole-grain bread, egg, milk, and flour</t>
         </is>
       </c>
       <c r="J169" s="22" t="n">

</xml_diff>

<commit_message>
Shaduled background, Update image
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="J75" s="9" t="n">
-        <v>3</v>
+        <v>3.05</v>
       </c>
       <c r="K75" s="15" t="n">
         <v>330</v>
@@ -8828,7 +8828,7 @@
         </is>
       </c>
       <c r="J125" s="9" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K125" s="15" t="n">
         <v>200</v>
@@ -8893,7 +8893,7 @@
         </is>
       </c>
       <c r="J126" s="9" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K126" s="15" t="n">
         <v>200</v>
@@ -8958,7 +8958,7 @@
         </is>
       </c>
       <c r="J127" s="9" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K127" s="15" t="n">
         <v>200</v>
@@ -9053,7 +9053,7 @@
         <v>0</v>
       </c>
       <c r="Q128" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R128" t="inlineStr">
         <is>
@@ -11129,7 +11129,11 @@
           <t>g</t>
         </is>
       </c>
-      <c r="M157" s="2" t="n"/>
+      <c r="M157" s="2" t="inlineStr">
+        <is>
+          <t>food/salads/buratina.jpg</t>
+        </is>
+      </c>
       <c r="N157" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat: translate Glarus beer descriptions to English, mark Pale Ale as recommended
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -1139,7 +1139,7 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
       <c r="J11" s="10" t="n">
-        <v>1</v>
+        <v>1.02</v>
       </c>
       <c r="K11" s="16" t="n">
         <v>70</v>
@@ -5782,6 +5782,20 @@
 Храна: универсална употреба</t>
         </is>
       </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>A pale beer brewed using traditional "ale" technology. Popular in the UK and the US among craft beer lovers for the countless possible combinations of hops and malt that lead to fascinating results. In our version we've used American and Slovenian hops, which complement each other perfectly and give a fresh citrus feel. We'll quench any thirst.
+Style: Pale Ale
+ABV: 4.2%
+Ingredients: water, 3 types of pale aromatic malt, 2 types of hops, brewer's yeast
+Color: golden
+Aroma: citrus fruits
+Taste: balanced; dry finish
+Body: light, medium-high carbonation
+Recommended serving temperature: 7-10°C
+Food pairing: versatile, pairs with everything</t>
+        </is>
+      </c>
       <c r="J82" s="9" t="n">
         <v>3.3</v>
       </c>
@@ -5805,7 +5819,7 @@
         <v>0</v>
       </c>
       <c r="P82" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q82" t="b">
         <v>1</v>
@@ -5867,6 +5881,21 @@
 Храна: универсална употреба</t>
         </is>
       </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Special English Ale - the most popular and beloved beer in England. A true classic! Perhaps the most widespread beer style in the UK.
+Stylistically, our "Special Ale" corresponds to the English "best/premium/special ale" category. The name comes from the quantity and quality of the raw materials used, as well as the alcohol content, which is slightly higher than an "ordinary bitter". This is an exceptionally easy-drinking beer you can enjoy any time.
+Style: Special/Best/Premium English Bitter
+ABV: 4.6%
+Ingredients: water, caramel and pale malt, 2 types of hops, brewer's yeast
+Color: deep golden/amber
+Aroma: caramel, fruity notes
+Taste: pleasantly crisp, lightly bitter; no sweetness lingers on the finish
+Body: medium body, medium-high carbonation
+Recommended serving temperature: 7-11°C
+Food pairing: versatile, pairs with everything</t>
+        </is>
+      </c>
       <c r="J83" s="9" t="n">
         <v>3.3</v>
       </c>
@@ -5889,8 +5918,8 @@
       <c r="O83" t="b">
         <v>0</v>
       </c>
-      <c r="P83" t="b">
-        <v>0</v>
+      <c r="P83" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="Q83" t="b">
         <v>1</v>
@@ -5954,6 +5983,23 @@
 Храна: сирена, пикантни ястия, ядки</t>
         </is>
       </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>IPA - the favorite drink of craft beer connoisseurs! A unique taste and aroma you'll remember!
+The IPA style was born out of necessity in 18th and 19th century England, which needed a beer that could survive the heat and long voyage to its distant colonies. The discovery that higher hopping significantly increased a beer's shelf life and stability sparked a true brewing revolution and delighted thirsty Englishmen around the world. Today the style is embraced by the craft industry across Europe and America, since it allows brewers to create truly unique, even extreme beers with fantastic aroma and complexity.
+Black Sea IPA by Glarus Craft Brewing is the first beer in our Glarus Signature series: an unfiltered beer with a unique character and no direct equivalent, combining Bulgarian hops, English brewer's yeast, and high-quality European malt into something we hope will impress even the most discerning craft beer connoisseurs.
+Product: Black Sea IPA
+Style: India Pale Ale (IPA)
+ABV: 6%
+Ingredients: water, malt, 2 types of hops, brewer's yeast
+Color: golden/light amber
+Aroma: citrus fruit, pine, and herbs
+Taste: refreshing, pleasantly bitter, a hint of caramel
+Body: medium body, medium-high carbonation
+Recommended serving temperature: 6-8°C
+Food pairing: cheeses, spicy dishes, nuts</t>
+        </is>
+      </c>
       <c r="J84" s="9" t="n">
         <v>3.3</v>
       </c>
@@ -5976,8 +6022,8 @@
       <c r="O84" t="b">
         <v>0</v>
       </c>
-      <c r="P84" t="b">
-        <v>0</v>
+      <c r="P84" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="Q84" t="b">
         <v>1</v>
@@ -6039,6 +6085,21 @@
 Храна: грил, сирена, летни ястия </t>
         </is>
       </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Based on the "Saison" style (literally "seasonal" beer), popular not only in Belgium but among craft brewers worldwide. We're fans too, because this style allows for quite a bit of "creative freedom" in the possible combinations of malt, hops, and spices. Still, there's one core rule we also follow - the beer should finish relatively dry, a result of using authentic Belgian yeast and a specific fermentation technique.
+Glarus SAISON is the perfect summer beer - fruity notes and a lightly peppery taste will invigorate and refresh you, while the dry finish helps quench your thirst.
+Style: Saison
+ABV: 5%
+Ingredients: water, malt, hops, cardamom, coriander, Belgian brewer's yeast
+Color: golden
+Aroma: delicate, with notes of exotic spices and orange
+Taste: matches the aroma, mellow alcohol, dry finish
+Body: medium-high
+Recommended serving temperature: 7-8°C
+Food pairing: grilled food, cheeses, summer dishes</t>
+        </is>
+      </c>
       <c r="J85" s="9" t="n">
         <v>3.3</v>
       </c>
@@ -6061,8 +6122,8 @@
       <c r="O85" t="b">
         <v>0</v>
       </c>
-      <c r="P85" t="b">
-        <v>0</v>
+      <c r="P85" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="Q85" t="b">
         <v>1</v>
@@ -6118,6 +6179,17 @@
 Сервиране: 6-8 С
 Цвят: 42 EBC
 Състав: вода, малц, мая, хмел, лешников екстракт</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>A dark ale combining five types of malt with the unmistakable aroma of toasted nuts and hazelnut!
+ABV: 5.5%
+Original gravity: 13°P
+IBU: 20
+Serving temperature: 6-8°C
+Color: 42 EBC
+Ingredients: water, malt, yeast, hops, hazelnut extract</t>
         </is>
       </c>
       <c r="J86" s="9" t="n">
@@ -6208,6 +6280,29 @@
 Храна: зрели сирена, червени меса, дивеч, печени меса, шоколадови и карамелени десерти</t>
         </is>
       </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Glarus Dubbel - when tradition has character
+Limited series
+Style: Dubbel / Abbey Ale
+ABV: 6.5%
+Some beers are meant to be drunk.
+Some beers are meant to be remembered.
+Glarus Dubbel is an abbey-style beer inspired by classic Belgian monastic brewing traditions - rich, aromatic, and made for people who want more than just a beer. Its deep dark amber color hides a rich aroma of caramel, dark malt, and dried fruit. The taste is smooth and balanced, with notes of raisins, figs, and brown sugar, finishing with a warm, velvety close. With its 6.5% ABV and 500 ml format, Glarus Dubbel offers a full-bodied experience and excellent value. A limited series, made to be shared, paired with food, and remembered. Glarus Dubbel. Abbey style. Limited series. True character.
+Glarus Dubbel is an abbey-style beer inspired by classic Belgian monastic brewing traditions.
+A limited series with a rich malt profile, smooth taste, and excellent drinkability.
+Distinguished by a deep dark amber to brown color, aromas of caramel, dark malt, and dried fruit, and a balanced, lightly sweet taste with a warm finish.
+Style: Dubbel
+ABV: 6.5%
+Ingredients: malt, hops, muscovado sugar, Belgian brewer's yeast, water
+Color: dark amber to brown, with a creamy head
+Aroma: caramel, dark malt, dried fruit, light spice notes
+Taste: raisins, figs, brown sugar, caramel
+Body: medium to full body, soft and smooth
+Recommended serving temperature: 8-10°C
+Food pairing: aged cheeses, red meats, game, roasted meats, chocolate and caramel desserts</t>
+        </is>
+      </c>
       <c r="J87" s="9" t="n">
         <v>3.3</v>
       </c>
@@ -6286,6 +6381,21 @@
 Плътност: средно плътно тяло, средна карбонизация
 Препоръчана температура на поднасяне: 7-12 градуса
 Храна: широк набор от месни храни и сирена</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Porter - inspired by the historic Porter style, known and loved by Londoners for several hundred years!
+Brown porter historically originated as a blend of different ales made purely from English ingredients. The flavor balance leans toward the malt, rather than the hops. We offer you magic in a deep brown color, with ruby highlights, good clarity, and a creamy head. A wonderful drink for cold days and nights. Limited batch.
+Style: Brown Porter
+ABV: 5.0%
+Ingredients: water, dark and pale malt, 2 types of hops, brewer's yeast
+Color: brown
+Aroma: caramel/chocolate with a hint of roasted nuts
+Taste: rich, lightly bitter
+Body: medium body, medium carbonation
+Recommended serving temperature: 7-12°C
+Food pairing: a wide range of meat dishes and cheeses</t>
         </is>
       </c>
       <c r="J88" s="9" t="n">

</xml_diff>

<commit_message>
some change in the ingredients of some of the items
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -5551,12 +5551,12 @@
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>хляб, моцарела, маслини</t>
+          <t>хляб, моцарела, маслини, сушен домат, подправки</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
         <is>
-          <t>bread, mozzarella, olives</t>
+          <t>bread, mozzarella, olives, sun-dried tomato, herbs</t>
         </is>
       </c>
       <c r="J79" s="18" t="n">

</xml_diff>

<commit_message>
feat: add lokum-web-v2 test container for v2.0 development
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1725" uniqueCount="928">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1727" uniqueCount="930">
   <si>
     <t>id</t>
   </si>
@@ -2952,6 +2952,12 @@
   </si>
   <si>
     <t>Sulphur dioxide and sulphites (preservatives, e.g. in wine).</t>
+  </si>
+  <si>
+    <t>cocktails/lokum/lokum.jpg</t>
+  </si>
+  <si>
+    <t>cocktails/nudistki_plazh.jpg</t>
   </si>
 </sst>
 </file>
@@ -8975,7 +8981,9 @@
       <c r="L114" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M114" s="2"/>
+      <c r="M114" s="2" t="s">
+        <v>928</v>
+      </c>
       <c r="N114" s="2" t="b">
         <v>0</v>
       </c>
@@ -9128,7 +9136,9 @@
       <c r="L117" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M117" s="2"/>
+      <c r="M117" s="2" t="s">
+        <v>929</v>
+      </c>
       <c r="N117" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add photos / update menu.json
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -2954,10 +2954,10 @@
     <t>Sulphur dioxide and sulphites (preservatives, e.g. in wine).</t>
   </si>
   <si>
-    <t>cocktails/lokum/lokum.jpg</t>
-  </si>
-  <si>
     <t>cocktails/nudistki_plazh.jpg</t>
+  </si>
+  <si>
+    <t>cocktails/lokum.jpg</t>
   </si>
 </sst>
 </file>
@@ -8258,7 +8258,7 @@
         <v>3.6</v>
       </c>
       <c r="K100" s="16">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="L100" s="2" t="s">
         <v>24</v>
@@ -8309,7 +8309,7 @@
         <v>3.6</v>
       </c>
       <c r="K101" s="16">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="L101" s="2" t="s">
         <v>24</v>
@@ -8982,7 +8982,7 @@
         <v>24</v>
       </c>
       <c r="M114" s="2" t="s">
-        <v>928</v>
+        <v>929</v>
       </c>
       <c r="N114" s="2" t="b">
         <v>0</v>
@@ -9137,7 +9137,7 @@
         <v>24</v>
       </c>
       <c r="M117" s="2" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="N117" s="2" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Add non-alcoholic cocktails and background to events button
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1727" uniqueCount="930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1738" uniqueCount="935">
   <si>
     <t>id</t>
   </si>
@@ -2958,6 +2958,21 @@
   </si>
   <si>
     <t>cocktails/lokum.jpg</t>
+  </si>
+  <si>
+    <t>Кокосов шейк</t>
+  </si>
+  <si>
+    <t>shake_coconut</t>
+  </si>
+  <si>
+    <t>Shake Coconut</t>
+  </si>
+  <si>
+    <t>Сироп кокос, мляко, сладолед</t>
+  </si>
+  <si>
+    <t>Coconut syrup, milk, ice cream</t>
   </si>
 </sst>
 </file>
@@ -3433,7 +3448,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S182"/>
+  <dimension ref="A1:S183"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.77734375" customWidth="1"/>
@@ -3453,7 +3468,7 @@
     <col min="15" max="15" width="8" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
     <col min="17" max="17" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="40.44140625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9681,10 +9696,10 @@
         <v>595</v>
       </c>
       <c r="J128" s="9">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K128" s="15">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L128" t="s">
         <v>24</v>
@@ -9699,7 +9714,7 @@
         <v>0</v>
       </c>
       <c r="Q128" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R128" t="s">
         <v>596</v>
@@ -9734,10 +9749,10 @@
         <v>601</v>
       </c>
       <c r="J129" s="9">
-        <v>4</v>
+        <v>3.3</v>
       </c>
       <c r="K129" s="15">
-        <v>330</v>
+        <v>200</v>
       </c>
       <c r="L129" t="s">
         <v>24</v>
@@ -9787,10 +9802,10 @@
         <v>605</v>
       </c>
       <c r="J130" s="9">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K130" s="15">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L130" t="s">
         <v>24</v>
@@ -9840,10 +9855,10 @@
         <v>610</v>
       </c>
       <c r="J131" s="9">
-        <v>4</v>
+        <v>3.8</v>
       </c>
       <c r="K131" s="15">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L131" t="s">
         <v>24</v>
@@ -10772,10 +10787,10 @@
         <v>700</v>
       </c>
       <c r="J149" s="9">
-        <v>5</v>
+        <v>3.8</v>
       </c>
       <c r="K149" s="15">
-        <v>330</v>
+        <v>200</v>
       </c>
       <c r="L149" t="s">
         <v>24</v>
@@ -10798,7 +10813,7 @@
     </row>
     <row r="150" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>701</v>
+        <v>931</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>342</v>
@@ -10810,25 +10825,25 @@
         <v>323</v>
       </c>
       <c r="E150" t="s">
-        <v>701</v>
+        <v>696</v>
       </c>
       <c r="F150" t="s">
-        <v>702</v>
+        <v>930</v>
       </c>
       <c r="G150" t="s">
-        <v>703</v>
+        <v>932</v>
       </c>
       <c r="H150" t="s">
-        <v>704</v>
+        <v>933</v>
       </c>
       <c r="I150" t="s">
-        <v>705</v>
+        <v>934</v>
       </c>
       <c r="J150" s="9">
-        <v>5</v>
+        <v>3.3</v>
       </c>
       <c r="K150" s="15">
-        <v>330</v>
+        <v>200</v>
       </c>
       <c r="L150" t="s">
         <v>24</v>
@@ -10851,7 +10866,7 @@
     </row>
     <row r="151" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>342</v>
@@ -10863,19 +10878,19 @@
         <v>323</v>
       </c>
       <c r="E151" t="s">
-        <v>706</v>
+        <v>701</v>
       </c>
       <c r="F151" t="s">
-        <v>707</v>
+        <v>702</v>
       </c>
       <c r="G151" t="s">
-        <v>708</v>
+        <v>703</v>
       </c>
       <c r="H151" t="s">
-        <v>709</v>
+        <v>704</v>
       </c>
       <c r="I151" t="s">
-        <v>710</v>
+        <v>705</v>
       </c>
       <c r="J151" s="9">
         <v>5</v>
@@ -10886,9 +10901,6 @@
       <c r="L151" t="s">
         <v>24</v>
       </c>
-      <c r="M151" t="s">
-        <v>711</v>
-      </c>
       <c r="N151" s="2" t="b">
         <v>0</v>
       </c>
@@ -10907,7 +10919,7 @@
     </row>
     <row r="152" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>712</v>
+        <v>706</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>342</v>
@@ -10919,19 +10931,19 @@
         <v>323</v>
       </c>
       <c r="E152" t="s">
-        <v>712</v>
+        <v>706</v>
       </c>
       <c r="F152" t="s">
-        <v>713</v>
+        <v>707</v>
       </c>
       <c r="G152" t="s">
-        <v>714</v>
+        <v>708</v>
       </c>
       <c r="H152" t="s">
-        <v>715</v>
+        <v>709</v>
       </c>
       <c r="I152" t="s">
-        <v>716</v>
+        <v>710</v>
       </c>
       <c r="J152" s="9">
         <v>5</v>
@@ -10942,6 +10954,9 @@
       <c r="L152" t="s">
         <v>24</v>
       </c>
+      <c r="M152" t="s">
+        <v>711</v>
+      </c>
       <c r="N152" s="2" t="b">
         <v>0</v>
       </c>
@@ -10960,7 +10975,7 @@
     </row>
     <row r="153" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>342</v>
@@ -10972,19 +10987,19 @@
         <v>323</v>
       </c>
       <c r="E153" t="s">
-        <v>717</v>
+        <v>712</v>
       </c>
       <c r="F153" t="s">
-        <v>718</v>
+        <v>713</v>
       </c>
       <c r="G153" t="s">
-        <v>719</v>
+        <v>714</v>
       </c>
       <c r="H153" t="s">
-        <v>720</v>
+        <v>715</v>
       </c>
       <c r="I153" t="s">
-        <v>721</v>
+        <v>716</v>
       </c>
       <c r="J153" s="9">
         <v>5</v>
@@ -11012,57 +11027,61 @@
       </c>
     </row>
     <row r="154" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A154" s="2" t="s">
+      <c r="A154" t="s">
+        <v>717</v>
+      </c>
+      <c r="B154" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C154" t="s">
+        <v>591</v>
+      </c>
+      <c r="D154" t="s">
+        <v>323</v>
+      </c>
+      <c r="E154" t="s">
+        <v>717</v>
+      </c>
+      <c r="F154" t="s">
+        <v>718</v>
+      </c>
+      <c r="G154" t="s">
+        <v>719</v>
+      </c>
+      <c r="H154" t="s">
+        <v>720</v>
+      </c>
+      <c r="I154" t="s">
+        <v>721</v>
+      </c>
+      <c r="J154" s="9">
+        <v>5</v>
+      </c>
+      <c r="K154" s="15">
+        <v>330</v>
+      </c>
+      <c r="L154" t="s">
+        <v>24</v>
+      </c>
+      <c r="N154" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O154" t="b">
+        <v>0</v>
+      </c>
+      <c r="P154" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q154" t="b">
+        <v>1</v>
+      </c>
+      <c r="R154" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="155" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A155" s="2" t="s">
         <v>722</v>
-      </c>
-      <c r="B154" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C154" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="D154" s="2"/>
-      <c r="E154" s="2"/>
-      <c r="F154" s="2" t="s">
-        <v>723</v>
-      </c>
-      <c r="G154" s="2" t="s">
-        <v>724</v>
-      </c>
-      <c r="H154" s="2"/>
-      <c r="I154" s="2"/>
-      <c r="J154" s="18">
-        <v>5.4</v>
-      </c>
-      <c r="K154" s="16">
-        <v>220</v>
-      </c>
-      <c r="L154" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="M154" s="2"/>
-      <c r="N154" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O154" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P154" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q154" t="b">
-        <v>1</v>
-      </c>
-      <c r="R154" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="S154" s="2" t="s">
-        <v>687</v>
-      </c>
-    </row>
-    <row r="155" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A155" s="2" t="s">
-        <v>725</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>47</v>
@@ -11073,29 +11092,23 @@
       <c r="D155" s="2"/>
       <c r="E155" s="2"/>
       <c r="F155" s="2" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>727</v>
-      </c>
-      <c r="H155" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="I155" s="2" t="s">
-        <v>729</v>
-      </c>
-      <c r="J155" s="8">
-        <v>5.6</v>
+        <v>724</v>
+      </c>
+      <c r="H155" s="2"/>
+      <c r="I155" s="2"/>
+      <c r="J155" s="18">
+        <v>5.4</v>
       </c>
       <c r="K155" s="16">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="L155" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M155" s="2" t="s">
-        <v>730</v>
-      </c>
+      <c r="M155" s="2"/>
       <c r="N155" s="2" t="b">
         <v>0</v>
       </c>
@@ -11112,12 +11125,12 @@
         <v>339</v>
       </c>
       <c r="S155" s="2" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="156" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="156" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>731</v>
+        <v>725</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>47</v>
@@ -11128,27 +11141,29 @@
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
       <c r="F156" s="2" t="s">
-        <v>732</v>
+        <v>726</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>733</v>
+        <v>727</v>
       </c>
       <c r="H156" s="2" t="s">
-        <v>734</v>
+        <v>728</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>735</v>
+        <v>729</v>
       </c>
       <c r="J156" s="8">
-        <v>6</v>
+        <v>5.6</v>
       </c>
       <c r="K156" s="16">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="L156" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M156" s="2"/>
+      <c r="M156" s="2" t="s">
+        <v>730</v>
+      </c>
       <c r="N156" s="2" t="b">
         <v>0</v>
       </c>
@@ -11158,52 +11173,50 @@
       <c r="P156" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q156" s="2" t="b">
-        <v>0</v>
+      <c r="Q156" t="b">
+        <v>1</v>
       </c>
       <c r="R156" s="2" t="s">
         <v>339</v>
       </c>
       <c r="S156" s="2" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="157" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="157" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>738</v>
+        <v>334</v>
       </c>
       <c r="D157" s="2"/>
       <c r="E157" s="2"/>
       <c r="F157" s="2" t="s">
-        <v>739</v>
+        <v>732</v>
       </c>
       <c r="G157" s="2" t="s">
-        <v>740</v>
+        <v>733</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>741</v>
+        <v>734</v>
       </c>
       <c r="I157" s="2" t="s">
-        <v>742</v>
-      </c>
-      <c r="J157" s="18">
+        <v>735</v>
+      </c>
+      <c r="J157" s="8">
         <v>6</v>
       </c>
       <c r="K157" s="16">
-        <v>330</v>
+        <v>240</v>
       </c>
       <c r="L157" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M157" s="2" t="s">
-        <v>743</v>
-      </c>
+      <c r="M157" s="2"/>
       <c r="N157" s="2" t="b">
         <v>0</v>
       </c>
@@ -11213,11 +11226,11 @@
       <c r="P157" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q157" t="b">
-        <v>1</v>
+      <c r="Q157" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R157" s="2" t="s">
-        <v>744</v>
+        <v>339</v>
       </c>
       <c r="S157" s="2" t="s">
         <v>736</v>
@@ -11225,39 +11238,39 @@
     </row>
     <row r="158" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
-        <v>745</v>
+        <v>737</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>672</v>
+        <v>738</v>
       </c>
       <c r="D158" s="2"/>
       <c r="E158" s="2"/>
       <c r="F158" s="2" t="s">
-        <v>746</v>
+        <v>739</v>
       </c>
       <c r="G158" s="2" t="s">
-        <v>747</v>
+        <v>740</v>
       </c>
       <c r="H158" s="2" t="s">
-        <v>748</v>
+        <v>741</v>
       </c>
       <c r="I158" s="2" t="s">
-        <v>749</v>
-      </c>
-      <c r="J158" s="8">
-        <v>6.4</v>
+        <v>742</v>
+      </c>
+      <c r="J158" s="18">
+        <v>6</v>
       </c>
       <c r="K158" s="16">
-        <v>400</v>
+        <v>330</v>
       </c>
       <c r="L158" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M158" s="2" t="s">
-        <v>750</v>
+        <v>743</v>
       </c>
       <c r="N158" s="2" t="b">
         <v>0</v>
@@ -11272,47 +11285,47 @@
         <v>1</v>
       </c>
       <c r="R158" s="2" t="s">
-        <v>677</v>
+        <v>744</v>
       </c>
       <c r="S158" s="2" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="159" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="159" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
-        <v>751</v>
+        <v>745</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>334</v>
+        <v>672</v>
       </c>
       <c r="D159" s="2"/>
       <c r="E159" s="2"/>
       <c r="F159" s="2" t="s">
-        <v>752</v>
+        <v>746</v>
       </c>
       <c r="G159" s="2" t="s">
-        <v>753</v>
+        <v>747</v>
       </c>
       <c r="H159" s="2" t="s">
-        <v>754</v>
+        <v>748</v>
       </c>
       <c r="I159" s="2" t="s">
-        <v>755</v>
+        <v>749</v>
       </c>
       <c r="J159" s="8">
-        <v>6.5</v>
+        <v>6.4</v>
       </c>
       <c r="K159" s="16">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="L159" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M159" s="2" t="s">
-        <v>756</v>
+        <v>750</v>
       </c>
       <c r="N159" s="2" t="b">
         <v>0</v>
@@ -11327,47 +11340,47 @@
         <v>1</v>
       </c>
       <c r="R159" s="2" t="s">
-        <v>339</v>
+        <v>677</v>
       </c>
       <c r="S159" s="2" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="160" spans="1:19" ht="138" customHeight="1" x14ac:dyDescent="0.3">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="160" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
-        <v>757</v>
+        <v>751</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>738</v>
+        <v>334</v>
       </c>
       <c r="D160" s="2"/>
       <c r="E160" s="2"/>
       <c r="F160" s="2" t="s">
-        <v>758</v>
+        <v>752</v>
       </c>
       <c r="G160" s="2" t="s">
-        <v>759</v>
+        <v>753</v>
       </c>
       <c r="H160" s="2" t="s">
-        <v>760</v>
+        <v>754</v>
       </c>
       <c r="I160" s="2" t="s">
-        <v>761</v>
-      </c>
-      <c r="J160" s="18">
-        <v>7.5</v>
+        <v>755</v>
+      </c>
+      <c r="J160" s="8">
+        <v>6.5</v>
       </c>
       <c r="K160" s="16">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L160" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M160" s="2" t="s">
-        <v>762</v>
+        <v>756</v>
       </c>
       <c r="N160" s="2" t="b">
         <v>0</v>
@@ -11382,47 +11395,47 @@
         <v>1</v>
       </c>
       <c r="R160" s="2" t="s">
-        <v>744</v>
+        <v>339</v>
       </c>
       <c r="S160" s="2" t="s">
-        <v>763</v>
-      </c>
-    </row>
-    <row r="161" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="161" spans="1:19" ht="138" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
-        <v>764</v>
+        <v>757</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C161" s="2" t="s">
-        <v>334</v>
+        <v>738</v>
       </c>
       <c r="D161" s="2"/>
       <c r="E161" s="2"/>
       <c r="F161" s="2" t="s">
-        <v>765</v>
+        <v>758</v>
       </c>
       <c r="G161" s="2" t="s">
-        <v>766</v>
+        <v>759</v>
       </c>
       <c r="H161" s="2" t="s">
-        <v>767</v>
+        <v>760</v>
       </c>
       <c r="I161" s="2" t="s">
-        <v>768</v>
-      </c>
-      <c r="J161" s="8">
-        <v>7.9</v>
+        <v>761</v>
+      </c>
+      <c r="J161" s="18">
+        <v>7.5</v>
       </c>
       <c r="K161" s="16">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="L161" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M161" s="2" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="N161" s="2" t="b">
         <v>0</v>
@@ -11437,15 +11450,15 @@
         <v>1</v>
       </c>
       <c r="R161" s="2" t="s">
-        <v>339</v>
+        <v>744</v>
       </c>
       <c r="S161" s="2" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="162" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="162" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>47</v>
@@ -11456,28 +11469,28 @@
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
       <c r="F162" s="2" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>772</v>
+        <v>766</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>773</v>
+        <v>767</v>
       </c>
       <c r="I162" s="2" t="s">
-        <v>774</v>
+        <v>768</v>
       </c>
       <c r="J162" s="8">
-        <v>9.5</v>
+        <v>7.9</v>
       </c>
       <c r="K162" s="16">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="L162" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M162" s="27" t="s">
-        <v>775</v>
+      <c r="M162" s="2" t="s">
+        <v>769</v>
       </c>
       <c r="N162" s="2" t="b">
         <v>0</v>
@@ -11495,56 +11508,67 @@
         <v>339</v>
       </c>
       <c r="S162" s="2" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="163" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A163" s="2" t="s">
+        <v>770</v>
+      </c>
+      <c r="B163" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C163" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="D163" s="2"/>
+      <c r="E163" s="2"/>
+      <c r="F163" s="2" t="s">
+        <v>771</v>
+      </c>
+      <c r="G163" s="2" t="s">
+        <v>772</v>
+      </c>
+      <c r="H163" s="2" t="s">
+        <v>773</v>
+      </c>
+      <c r="I163" s="2" t="s">
+        <v>774</v>
+      </c>
+      <c r="J163" s="8">
+        <v>9.5</v>
+      </c>
+      <c r="K163" s="16">
+        <v>250</v>
+      </c>
+      <c r="L163" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M163" s="27" t="s">
+        <v>775</v>
+      </c>
+      <c r="N163" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O163" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P163" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q163" t="b">
+        <v>1</v>
+      </c>
+      <c r="R163" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="S163" s="2" t="s">
         <v>63</v>
-      </c>
-    </row>
-    <row r="163" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A163" t="s">
-        <v>776</v>
-      </c>
-      <c r="B163" t="s">
-        <v>20</v>
-      </c>
-      <c r="C163" s="21" t="s">
-        <v>577</v>
-      </c>
-      <c r="D163" t="s">
-        <v>578</v>
-      </c>
-      <c r="E163" t="s">
-        <v>579</v>
-      </c>
-      <c r="F163" t="s">
-        <v>777</v>
-      </c>
-      <c r="G163" t="s">
-        <v>778</v>
-      </c>
-      <c r="J163" s="9">
-        <v>12</v>
-      </c>
-      <c r="K163" s="15">
-        <v>750</v>
-      </c>
-      <c r="L163" t="s">
-        <v>24</v>
-      </c>
-      <c r="O163" t="b">
-        <v>0</v>
-      </c>
-      <c r="P163" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q163" t="b">
-        <v>1</v>
-      </c>
-      <c r="R163" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="164" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>779</v>
+        <v>776</v>
       </c>
       <c r="B164" t="s">
         <v>20</v>
@@ -11556,13 +11580,13 @@
         <v>578</v>
       </c>
       <c r="E164" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="F164" t="s">
-        <v>780</v>
+        <v>777</v>
       </c>
       <c r="G164" t="s">
-        <v>781</v>
+        <v>778</v>
       </c>
       <c r="J164" s="9">
         <v>12</v>
@@ -11588,7 +11612,7 @@
     </row>
     <row r="165" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>782</v>
+        <v>779</v>
       </c>
       <c r="B165" t="s">
         <v>20</v>
@@ -11600,13 +11624,13 @@
         <v>578</v>
       </c>
       <c r="E165" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="F165" t="s">
-        <v>783</v>
+        <v>780</v>
       </c>
       <c r="G165" t="s">
-        <v>784</v>
+        <v>781</v>
       </c>
       <c r="J165" s="9">
         <v>12</v>
@@ -11630,87 +11654,80 @@
         <v>309</v>
       </c>
     </row>
-    <row r="166" spans="1:19" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A166" s="2" t="s">
+    <row r="166" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>782</v>
+      </c>
+      <c r="B166" t="s">
+        <v>20</v>
+      </c>
+      <c r="C166" s="21" t="s">
+        <v>577</v>
+      </c>
+      <c r="D166" t="s">
+        <v>578</v>
+      </c>
+      <c r="E166" t="s">
+        <v>587</v>
+      </c>
+      <c r="F166" t="s">
+        <v>783</v>
+      </c>
+      <c r="G166" t="s">
+        <v>784</v>
+      </c>
+      <c r="J166" s="9">
+        <v>12</v>
+      </c>
+      <c r="K166" s="15">
+        <v>750</v>
+      </c>
+      <c r="L166" t="s">
+        <v>24</v>
+      </c>
+      <c r="O166" t="b">
+        <v>0</v>
+      </c>
+      <c r="P166" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q166" t="b">
+        <v>1</v>
+      </c>
+      <c r="R166" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="167" spans="1:19" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A167" s="2" t="s">
         <v>785</v>
       </c>
-      <c r="B166" s="2" t="s">
+      <c r="B167" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C166" s="2" t="s">
+      <c r="C167" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D166" s="2"/>
-      <c r="E166" s="2"/>
-      <c r="F166" s="12" t="s">
+      <c r="D167" s="2"/>
+      <c r="E167" s="2"/>
+      <c r="F167" s="12" t="s">
         <v>786</v>
       </c>
-      <c r="G166" s="12" t="s">
+      <c r="G167" s="12" t="s">
         <v>787</v>
       </c>
-      <c r="H166" s="12" t="s">
+      <c r="H167" s="12" t="s">
         <v>788</v>
       </c>
-      <c r="I166" s="12" t="s">
+      <c r="I167" s="12" t="s">
         <v>789</v>
       </c>
-      <c r="J166" s="22"/>
-      <c r="K166" s="16">
-        <v>200</v>
-      </c>
-      <c r="L166" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="M166" s="2"/>
-      <c r="N166" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O166" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P166" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q166" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R166" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="S166" s="2" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="167" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A167" s="2" t="s">
-        <v>791</v>
-      </c>
-      <c r="B167" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C167" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D167" s="2" t="s">
-        <v>792</v>
-      </c>
-      <c r="E167" s="2" t="s">
-        <v>793</v>
-      </c>
-      <c r="F167" s="12" t="s">
-        <v>794</v>
-      </c>
-      <c r="G167" s="12" t="s">
-        <v>795</v>
-      </c>
-      <c r="H167" s="12"/>
-      <c r="I167" s="12"/>
       <c r="J167" s="22"/>
       <c r="K167" s="16">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="L167" s="2" t="s">
-        <v>24</v>
+        <v>61</v>
       </c>
       <c r="M167" s="2"/>
       <c r="N167" s="2" t="b">
@@ -11726,40 +11743,42 @@
         <v>0</v>
       </c>
       <c r="R167" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="S167" s="2"/>
-    </row>
-    <row r="168" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+        <v>339</v>
+      </c>
+      <c r="S167" s="2" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="168" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>796</v>
+        <v>791</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C168" s="2" t="s">
-        <v>672</v>
-      </c>
-      <c r="D168" s="2"/>
-      <c r="E168" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="C168" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D168" s="2" t="s">
+        <v>792</v>
+      </c>
+      <c r="E168" s="2" t="s">
+        <v>793</v>
+      </c>
       <c r="F168" s="12" t="s">
-        <v>797</v>
+        <v>794</v>
       </c>
       <c r="G168" s="12" t="s">
-        <v>798</v>
-      </c>
-      <c r="H168" s="12" t="s">
-        <v>799</v>
-      </c>
-      <c r="I168" s="12" t="s">
-        <v>800</v>
-      </c>
+        <v>795</v>
+      </c>
+      <c r="H168" s="12"/>
+      <c r="I168" s="12"/>
       <c r="J168" s="22"/>
       <c r="K168" s="16">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="L168" s="2" t="s">
-        <v>61</v>
+        <v>24</v>
       </c>
       <c r="M168" s="2"/>
       <c r="N168" s="2" t="b">
@@ -11775,15 +11794,13 @@
         <v>0</v>
       </c>
       <c r="R168" s="2" t="s">
-        <v>677</v>
-      </c>
-      <c r="S168" s="2" t="s">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="169" spans="1:19" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+      <c r="S168" s="2"/>
+    </row>
+    <row r="169" spans="1:19" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
-        <v>802</v>
+        <v>796</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>47</v>
@@ -11794,20 +11811,20 @@
       <c r="D169" s="2"/>
       <c r="E169" s="2"/>
       <c r="F169" s="12" t="s">
-        <v>803</v>
+        <v>797</v>
       </c>
       <c r="G169" s="12" t="s">
-        <v>804</v>
+        <v>798</v>
       </c>
       <c r="H169" s="12" t="s">
-        <v>805</v>
+        <v>799</v>
       </c>
       <c r="I169" s="12" t="s">
-        <v>806</v>
+        <v>800</v>
       </c>
       <c r="J169" s="22"/>
       <c r="K169" s="16">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="L169" s="2" t="s">
         <v>61</v>
@@ -11832,9 +11849,9 @@
         <v>801</v>
       </c>
     </row>
-    <row r="170" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:19" ht="39.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
-        <v>807</v>
+        <v>802</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>47</v>
@@ -11845,16 +11862,16 @@
       <c r="D170" s="2"/>
       <c r="E170" s="2"/>
       <c r="F170" s="12" t="s">
-        <v>808</v>
+        <v>803</v>
       </c>
       <c r="G170" s="12" t="s">
-        <v>809</v>
+        <v>804</v>
       </c>
       <c r="H170" s="12" t="s">
-        <v>810</v>
+        <v>805</v>
       </c>
       <c r="I170" s="12" t="s">
-        <v>811</v>
+        <v>806</v>
       </c>
       <c r="J170" s="22"/>
       <c r="K170" s="16">
@@ -11880,45 +11897,41 @@
         <v>677</v>
       </c>
       <c r="S170" s="2" t="s">
-        <v>812</v>
+        <v>801</v>
       </c>
     </row>
     <row r="171" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
-        <v>813</v>
+        <v>807</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>814</v>
+        <v>672</v>
       </c>
       <c r="D171" s="2"/>
       <c r="E171" s="2"/>
       <c r="F171" s="12" t="s">
-        <v>815</v>
+        <v>808</v>
       </c>
       <c r="G171" s="12" t="s">
-        <v>816</v>
+        <v>809</v>
       </c>
       <c r="H171" s="12" t="s">
-        <v>817</v>
+        <v>810</v>
       </c>
       <c r="I171" s="12" t="s">
-        <v>818</v>
-      </c>
-      <c r="J171" s="22">
-        <v>3.3</v>
-      </c>
+        <v>811</v>
+      </c>
+      <c r="J171" s="22"/>
       <c r="K171" s="16">
-        <v>270</v>
+        <v>280</v>
       </c>
       <c r="L171" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M171" s="2" t="s">
-        <v>819</v>
-      </c>
+      <c r="M171" s="2"/>
       <c r="N171" s="2" t="b">
         <v>0</v>
       </c>
@@ -11928,19 +11941,19 @@
       <c r="P171" s="2" t="b">
         <v>0</v>
       </c>
-      <c r="Q171" t="b">
-        <v>1</v>
+      <c r="Q171" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="R171" s="2" t="s">
-        <v>820</v>
+        <v>677</v>
       </c>
       <c r="S171" s="2" t="s">
-        <v>497</v>
+        <v>812</v>
       </c>
     </row>
     <row r="172" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
-        <v>821</v>
+        <v>813</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>47</v>
@@ -11951,28 +11964,28 @@
       <c r="D172" s="2"/>
       <c r="E172" s="2"/>
       <c r="F172" s="12" t="s">
-        <v>822</v>
+        <v>815</v>
       </c>
       <c r="G172" s="12" t="s">
-        <v>823</v>
+        <v>816</v>
       </c>
       <c r="H172" s="12" t="s">
-        <v>824</v>
+        <v>817</v>
       </c>
       <c r="I172" s="12" t="s">
-        <v>825</v>
+        <v>818</v>
       </c>
       <c r="J172" s="22">
-        <v>6.9</v>
+        <v>3.3</v>
       </c>
       <c r="K172" s="16">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="L172" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M172" s="2" t="s">
-        <v>826</v>
+        <v>819</v>
       </c>
       <c r="N172" s="2" t="b">
         <v>0</v>
@@ -11990,12 +12003,12 @@
         <v>820</v>
       </c>
       <c r="S172" s="2" t="s">
-        <v>827</v>
+        <v>497</v>
       </c>
     </row>
     <row r="173" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
-        <v>828</v>
+        <v>821</v>
       </c>
       <c r="B173" s="2" t="s">
         <v>47</v>
@@ -12006,28 +12019,28 @@
       <c r="D173" s="2"/>
       <c r="E173" s="2"/>
       <c r="F173" s="12" t="s">
-        <v>829</v>
+        <v>822</v>
       </c>
       <c r="G173" s="12" t="s">
-        <v>830</v>
+        <v>823</v>
       </c>
       <c r="H173" s="12" t="s">
-        <v>831</v>
+        <v>824</v>
       </c>
       <c r="I173" s="12" t="s">
-        <v>832</v>
+        <v>825</v>
       </c>
       <c r="J173" s="22">
-        <v>3.4</v>
+        <v>6.9</v>
       </c>
       <c r="K173" s="16">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="L173" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M173" s="2" t="s">
-        <v>833</v>
+        <v>826</v>
       </c>
       <c r="N173" s="2" t="b">
         <v>0</v>
@@ -12045,12 +12058,12 @@
         <v>820</v>
       </c>
       <c r="S173" s="2" t="s">
-        <v>497</v>
+        <v>827</v>
       </c>
     </row>
     <row r="174" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
-        <v>834</v>
+        <v>828</v>
       </c>
       <c r="B174" s="2" t="s">
         <v>47</v>
@@ -12061,28 +12074,28 @@
       <c r="D174" s="2"/>
       <c r="E174" s="2"/>
       <c r="F174" s="12" t="s">
-        <v>835</v>
+        <v>829</v>
       </c>
       <c r="G174" s="12" t="s">
-        <v>836</v>
+        <v>830</v>
       </c>
       <c r="H174" s="12" t="s">
-        <v>837</v>
+        <v>831</v>
       </c>
       <c r="I174" s="12" t="s">
-        <v>838</v>
+        <v>832</v>
       </c>
       <c r="J174" s="22">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="K174" s="16">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="L174" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M174" s="2" t="s">
-        <v>839</v>
+        <v>833</v>
       </c>
       <c r="N174" s="2" t="b">
         <v>0</v>
@@ -12099,13 +12112,13 @@
       <c r="R174" s="2" t="s">
         <v>820</v>
       </c>
-      <c r="S174" s="25" t="s">
-        <v>340</v>
+      <c r="S174" s="2" t="s">
+        <v>497</v>
       </c>
     </row>
     <row r="175" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
-        <v>840</v>
+        <v>834</v>
       </c>
       <c r="B175" s="2" t="s">
         <v>47</v>
@@ -12116,28 +12129,28 @@
       <c r="D175" s="2"/>
       <c r="E175" s="2"/>
       <c r="F175" s="12" t="s">
-        <v>841</v>
+        <v>835</v>
       </c>
       <c r="G175" s="12" t="s">
-        <v>842</v>
+        <v>836</v>
       </c>
       <c r="H175" s="12" t="s">
-        <v>843</v>
+        <v>837</v>
       </c>
       <c r="I175" s="12" t="s">
-        <v>844</v>
+        <v>838</v>
       </c>
       <c r="J175" s="22">
-        <v>4.9000000000000004</v>
+        <v>3.1</v>
       </c>
       <c r="K175" s="16">
-        <v>270</v>
+        <v>400</v>
       </c>
       <c r="L175" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M175" s="2" t="s">
-        <v>845</v>
+        <v>839</v>
       </c>
       <c r="N175" s="2" t="b">
         <v>0</v>
@@ -12155,12 +12168,12 @@
         <v>820</v>
       </c>
       <c r="S175" s="25" t="s">
-        <v>687</v>
+        <v>340</v>
       </c>
     </row>
     <row r="176" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
-        <v>846</v>
+        <v>840</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>47</v>
@@ -12171,22 +12184,28 @@
       <c r="D176" s="2"/>
       <c r="E176" s="2"/>
       <c r="F176" s="12" t="s">
-        <v>847</v>
+        <v>841</v>
       </c>
       <c r="G176" s="12" t="s">
-        <v>848</v>
-      </c>
-      <c r="H176" s="12"/>
-      <c r="I176" s="12"/>
+        <v>842</v>
+      </c>
+      <c r="H176" s="12" t="s">
+        <v>843</v>
+      </c>
+      <c r="I176" s="12" t="s">
+        <v>844</v>
+      </c>
       <c r="J176" s="22">
-        <v>6.5</v>
-      </c>
-      <c r="K176" s="16"/>
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="K176" s="16">
+        <v>270</v>
+      </c>
       <c r="L176" s="2" t="s">
         <v>61</v>
       </c>
       <c r="M176" s="2" t="s">
-        <v>849</v>
+        <v>845</v>
       </c>
       <c r="N176" s="2" t="b">
         <v>0</v>
@@ -12204,121 +12223,129 @@
         <v>820</v>
       </c>
       <c r="S176" s="25" t="s">
-        <v>850</v>
-      </c>
-    </row>
-    <row r="177" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="177" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
-        <v>851</v>
+        <v>846</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>342</v>
+        <v>47</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>343</v>
+        <v>814</v>
       </c>
       <c r="D177" s="2"/>
       <c r="E177" s="2"/>
       <c r="F177" s="12" t="s">
+        <v>847</v>
+      </c>
+      <c r="G177" s="12" t="s">
+        <v>848</v>
+      </c>
+      <c r="H177" s="12"/>
+      <c r="I177" s="12"/>
+      <c r="J177" s="22">
+        <v>6.5</v>
+      </c>
+      <c r="K177" s="16"/>
+      <c r="L177" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="M177" s="2" t="s">
+        <v>849</v>
+      </c>
+      <c r="N177" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O177" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P177" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q177" t="b">
+        <v>1</v>
+      </c>
+      <c r="R177" s="2" t="s">
+        <v>820</v>
+      </c>
+      <c r="S177" s="25" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="178" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A178" s="2" t="s">
+        <v>851</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="D178" s="2"/>
+      <c r="E178" s="2"/>
+      <c r="F178" s="12" t="s">
         <v>852</v>
       </c>
-      <c r="G177" s="12" t="s">
+      <c r="G178" s="12" t="s">
         <v>853</v>
       </c>
-      <c r="H177" s="12" t="s">
+      <c r="H178" s="12" t="s">
         <v>854</v>
       </c>
-      <c r="I177" s="12" t="s">
+      <c r="I178" s="12" t="s">
         <v>855</v>
       </c>
-      <c r="J177" s="22">
+      <c r="J178" s="22">
         <v>3.3</v>
       </c>
-      <c r="K177" s="20">
+      <c r="K178" s="20">
         <v>150</v>
       </c>
-      <c r="L177" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M177" s="2"/>
-      <c r="N177" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O177" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P177" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q177" t="b">
-        <v>1</v>
-      </c>
-      <c r="R177" s="2" t="s">
+      <c r="L178" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M178" s="2"/>
+      <c r="N178" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O178" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P178" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q178" t="b">
+        <v>1</v>
+      </c>
+      <c r="R178" s="2" t="s">
         <v>856</v>
       </c>
-      <c r="S177" s="2"/>
-    </row>
-    <row r="178" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A178" t="s">
-        <v>857</v>
-      </c>
-      <c r="B178" t="s">
-        <v>20</v>
-      </c>
-      <c r="C178" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="F178" s="13" t="s">
-        <v>858</v>
-      </c>
-      <c r="G178" s="13" t="s">
-        <v>859</v>
-      </c>
-      <c r="H178" s="13"/>
-      <c r="I178" s="13"/>
-      <c r="J178" s="22">
-        <v>3.1</v>
-      </c>
-      <c r="K178" s="15"/>
-      <c r="L178" t="s">
-        <v>24</v>
-      </c>
-      <c r="N178" t="b">
-        <v>0</v>
-      </c>
-      <c r="O178" t="b">
-        <v>0</v>
-      </c>
-      <c r="P178" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q178" t="b">
-        <v>1</v>
-      </c>
-      <c r="R178" t="s">
-        <v>25</v>
-      </c>
+      <c r="S178" s="2"/>
     </row>
     <row r="179" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>860</v>
+        <v>857</v>
       </c>
       <c r="B179" t="s">
         <v>20</v>
       </c>
       <c r="C179" s="21" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F179" s="13" t="s">
-        <v>861</v>
+        <v>858</v>
       </c>
       <c r="G179" s="13" t="s">
-        <v>862</v>
+        <v>859</v>
       </c>
       <c r="H179" s="13"/>
       <c r="I179" s="13"/>
       <c r="J179" s="22">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
       <c r="K179" s="15"/>
       <c r="L179" t="s">
@@ -12342,7 +12369,7 @@
     </row>
     <row r="180" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>863</v>
+        <v>860</v>
       </c>
       <c r="B180" t="s">
         <v>20</v>
@@ -12350,18 +12377,21 @@
       <c r="C180" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="F180" s="14" t="s">
-        <v>864</v>
+      <c r="F180" s="13" t="s">
+        <v>861</v>
       </c>
       <c r="G180" s="13" t="s">
-        <v>865</v>
+        <v>862</v>
       </c>
       <c r="H180" s="13"/>
       <c r="I180" s="13"/>
       <c r="J180" s="22">
-        <v>0.35</v>
+        <v>1.8</v>
       </c>
       <c r="K180" s="15"/>
+      <c r="L180" t="s">
+        <v>24</v>
+      </c>
       <c r="N180" t="b">
         <v>0</v>
       </c>
@@ -12380,34 +12410,26 @@
     </row>
     <row r="181" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>866</v>
+        <v>863</v>
       </c>
       <c r="B181" t="s">
         <v>20</v>
       </c>
-      <c r="C181" t="s">
-        <v>65</v>
-      </c>
-      <c r="D181" t="s">
-        <v>133</v>
-      </c>
-      <c r="F181" s="13" t="s">
-        <v>134</v>
+      <c r="C181" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F181" s="14" t="s">
+        <v>864</v>
       </c>
       <c r="G181" s="13" t="s">
-        <v>135</v>
+        <v>865</v>
       </c>
       <c r="H181" s="13"/>
       <c r="I181" s="13"/>
       <c r="J181" s="22">
-        <v>1</v>
-      </c>
-      <c r="K181" s="15">
-        <v>500</v>
-      </c>
-      <c r="L181" t="s">
-        <v>24</v>
-      </c>
+        <v>0.35</v>
+      </c>
+      <c r="K181" s="15"/>
       <c r="N181" t="b">
         <v>0</v>
       </c>
@@ -12426,7 +12448,7 @@
     </row>
     <row r="182" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>867</v>
+        <v>866</v>
       </c>
       <c r="B182" t="s">
         <v>20</v>
@@ -12434,36 +12456,82 @@
       <c r="C182" t="s">
         <v>65</v>
       </c>
+      <c r="D182" t="s">
+        <v>133</v>
+      </c>
       <c r="F182" s="13" t="s">
-        <v>868</v>
+        <v>134</v>
       </c>
       <c r="G182" s="13" t="s">
-        <v>869</v>
+        <v>135</v>
       </c>
       <c r="H182" s="13"/>
       <c r="I182" s="13"/>
       <c r="J182" s="22">
+        <v>1</v>
+      </c>
+      <c r="K182" s="15">
+        <v>500</v>
+      </c>
+      <c r="L182" t="s">
+        <v>24</v>
+      </c>
+      <c r="N182" t="b">
+        <v>0</v>
+      </c>
+      <c r="O182" t="b">
+        <v>0</v>
+      </c>
+      <c r="P182" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q182" t="b">
+        <v>1</v>
+      </c>
+      <c r="R182" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="183" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>867</v>
+      </c>
+      <c r="B183" t="s">
+        <v>20</v>
+      </c>
+      <c r="C183" t="s">
+        <v>65</v>
+      </c>
+      <c r="F183" s="13" t="s">
+        <v>868</v>
+      </c>
+      <c r="G183" s="13" t="s">
+        <v>869</v>
+      </c>
+      <c r="H183" s="13"/>
+      <c r="I183" s="13"/>
+      <c r="J183" s="22">
         <v>4.0999999999999996</v>
       </c>
-      <c r="K182" s="15">
+      <c r="K183" s="15">
         <v>200</v>
       </c>
-      <c r="L182" t="s">
-        <v>24</v>
-      </c>
-      <c r="N182" t="b">
-        <v>0</v>
-      </c>
-      <c r="O182" t="b">
-        <v>0</v>
-      </c>
-      <c r="P182" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q182" t="b">
-        <v>1</v>
-      </c>
-      <c r="R182" t="s">
+      <c r="L183" t="s">
+        <v>24</v>
+      </c>
+      <c r="N183" t="b">
+        <v>0</v>
+      </c>
+      <c r="O183" t="b">
+        <v>0</v>
+      </c>
+      <c r="P183" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q183" t="b">
+        <v>1</v>
+      </c>
+      <c r="R183" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Compress photos, fix wine/pks image paths, add missed ISHTAH event
- Re-compressed nearly all bundled images (products_master.xlsx source updated too)
- menu.json: wine/cheval_chardonnay_750.jpg and food/mains/pks.jpg were pointing
  at nonexistent default .webp paths - fixed to the real bundled files
- events.json: added the missed ISHTAH exhibition (Emilia Baleva, 2025-11-15)
- pubspec.yaml: declared the new events/archive/ishtah/ asset folder
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1738" uniqueCount="935">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1740" uniqueCount="937">
   <si>
     <t>id</t>
   </si>
@@ -2973,6 +2973,12 @@
   </si>
   <si>
     <t>Coconut syrup, milk, ice cream</t>
+  </si>
+  <si>
+    <t>food/mains/pks.jpg</t>
+  </si>
+  <si>
+    <t>wine/cheval_chardonnay_750.jpg</t>
   </si>
 </sst>
 </file>
@@ -3463,7 +3469,7 @@
     <col min="10" max="10" width="10" style="4" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
     <col min="12" max="12" width="8" customWidth="1"/>
-    <col min="13" max="13" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="26.77734375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="9" customWidth="1"/>
     <col min="15" max="15" width="8" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
@@ -10067,7 +10073,9 @@
       <c r="L135" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M135" s="2"/>
+      <c r="M135" s="2" t="s">
+        <v>935</v>
+      </c>
       <c r="N135" s="2" t="b">
         <v>0</v>
       </c>
@@ -11566,7 +11574,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="164" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>776</v>
       </c>
@@ -11596,6 +11604,9 @@
       </c>
       <c r="L164" t="s">
         <v>24</v>
+      </c>
+      <c r="M164" s="2" t="s">
+        <v>936</v>
       </c>
       <c r="O164" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
Fix acoustic_adventures gallery mix-up, add brusketi_s_proshuto photo
The two Acoustic Adventures #1 gallery photos had been moved into the #2
event's folder by mistake - moved back to part1/, and part2 now has its
own actual gallery photo instead of borrowing part1's.

menu.json: brusketi_s_proshuto was pointing at the nonexistent default
.webp path - fixed to the real bundled food/mains/brusketi_s_proshuto.jpg.
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1740" uniqueCount="937">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="938">
   <si>
     <t>id</t>
   </si>
@@ -2979,6 +2979,9 @@
   </si>
   <si>
     <t>wine/cheval_chardonnay_750.jpg</t>
+  </si>
+  <si>
+    <t>food/mains/brusketi_s_proshuto.jpg</t>
   </si>
 </sst>
 </file>
@@ -10126,7 +10129,9 @@
       <c r="L136" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="M136" s="2"/>
+      <c r="M136" s="2" t="s">
+        <v>937</v>
+      </c>
       <c r="N136" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Update products_master.xlsx with aperol image path
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1742" uniqueCount="939">
   <si>
     <t>id</t>
   </si>
@@ -2982,6 +2982,9 @@
   </si>
   <si>
     <t>food/mains/brusketi_s_proshuto.jpg</t>
+  </si>
+  <si>
+    <t>cocktails/aperol.jpg</t>
   </si>
 </sst>
 </file>
@@ -6101,7 +6104,9 @@
       <c r="L57" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M57" s="2"/>
+      <c r="M57" s="2" t="s">
+        <v>938</v>
+      </c>
       <c r="N57" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Sync products_master.xlsx: aperol.jpg belongs to Aperol Spritz row
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -6104,9 +6104,7 @@
       <c r="L57" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M57" s="2" t="s">
-        <v>938</v>
-      </c>
+      <c r="M57" s="2"/>
       <c r="N57" s="2" t="b">
         <v>0</v>
       </c>
@@ -9371,7 +9369,9 @@
       <c r="L121" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M121" s="2"/>
+      <c r="M121" s="2" t="s">
+        <v>938</v>
+      </c>
       <c r="N121" s="2" t="b">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Add blueberry cheesecake to desserts, marked new and pinned to top
Manual menu.json patch (not regenerated from excel) to ship before
brunch - the excel itself doesn't have this row yet, so it will
disappear on the next excel_to_json.py regen unless added there too.
Price/weight (4.80 EUR, 150g) and allergens are a best guess from the
closest existing dessert (torta_lokum) - please confirm.
</commit_message>
<xml_diff>
--- a/database/excel/products_master.xlsx
+++ b/database/excel/products_master.xlsx
@@ -11,14 +11,14 @@
     <sheet name="allergens" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">products!$A$1:$S$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">products!$A$1:$S$122</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1710" uniqueCount="922">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1719" uniqueCount="927">
   <si>
     <t>id</t>
   </si>
@@ -2934,6 +2934,21 @@
   </si>
   <si>
     <t xml:space="preserve">3 in 1 </t>
+  </si>
+  <si>
+    <t>Боровинков чийзкейк</t>
+  </si>
+  <si>
+    <t>Blueberry cheesecake</t>
+  </si>
+  <si>
+    <t>1,3,7,9</t>
+  </si>
+  <si>
+    <t>borovinkov_cheese_cake</t>
+  </si>
+  <si>
+    <t>food/desserts/borovinkov_cheese_cake.jpg</t>
   </si>
 </sst>
 </file>
@@ -3409,7 +3424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S185"/>
+  <dimension ref="A1:S186"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.77734375" customWidth="1"/>
@@ -8280,34 +8295,36 @@
     </row>
     <row r="103" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
-        <v>376</v>
+        <v>925</v>
       </c>
       <c r="B103" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>292</v>
+        <v>54</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
       <c r="F103" s="2" t="s">
-        <v>377</v>
+        <v>922</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>378</v>
+        <v>923</v>
       </c>
       <c r="H103" s="2"/>
       <c r="I103" s="2"/>
-      <c r="J103" s="18">
-        <v>3.6</v>
+      <c r="J103" s="8">
+        <v>4.5</v>
       </c>
       <c r="K103" s="16">
-        <v>300</v>
+        <v>180</v>
       </c>
       <c r="L103" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M103" s="2"/>
+      <c r="M103" s="2" t="s">
+        <v>926</v>
+      </c>
       <c r="N103" s="2" t="b">
         <v>0</v>
       </c>
@@ -8321,42 +8338,40 @@
         <v>1</v>
       </c>
       <c r="R103" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S103" s="2"/>
+        <v>58</v>
+      </c>
+      <c r="S103" s="2" t="s">
+        <v>924</v>
+      </c>
     </row>
     <row r="104" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D104" s="2" t="s">
-        <v>380</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>292</v>
+      </c>
+      <c r="D104" s="2"/>
+      <c r="E104" s="2"/>
       <c r="F104" s="2" t="s">
-        <v>880</v>
+        <v>377</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="H104" s="2"/>
       <c r="I104" s="2"/>
-      <c r="J104" s="8">
-        <v>3.9</v>
+      <c r="J104" s="18">
+        <v>3.6</v>
       </c>
       <c r="K104" s="16">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="L104" s="2" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="M104" s="2"/>
       <c r="N104" s="2" t="b">
@@ -8372,39 +8387,39 @@
         <v>1</v>
       </c>
       <c r="R104" s="2" t="s">
-        <v>382</v>
+        <v>297</v>
       </c>
       <c r="S104" s="2"/>
     </row>
     <row r="105" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>300</v>
+        <v>20</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D105" s="2"/>
-      <c r="E105" s="2"/>
+        <v>65</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="F105" s="2" t="s">
-        <v>385</v>
+        <v>880</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="H105" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="I105" s="2" t="s">
-        <v>388</v>
-      </c>
+        <v>381</v>
+      </c>
+      <c r="H105" s="2"/>
+      <c r="I105" s="2"/>
       <c r="J105" s="8">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="K105" s="16">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="L105" s="2" t="s">
         <v>24</v>
@@ -8423,15 +8438,13 @@
         <v>1</v>
       </c>
       <c r="R105" s="2" t="s">
-        <v>389</v>
-      </c>
-      <c r="S105" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="106" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>382</v>
+      </c>
+      <c r="S105" s="2"/>
+    </row>
+    <row r="106" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
-        <v>390</v>
+        <v>383</v>
       </c>
       <c r="B106" s="2" t="s">
         <v>300</v>
@@ -8442,22 +8455,22 @@
       <c r="D106" s="2"/>
       <c r="E106" s="2"/>
       <c r="F106" s="2" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="H106" s="2" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="I106" s="2" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="J106" s="8">
         <v>4</v>
       </c>
       <c r="K106" s="16">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="L106" s="2" t="s">
         <v>24</v>
@@ -8476,13 +8489,15 @@
         <v>1</v>
       </c>
       <c r="R106" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="S106" s="2"/>
-    </row>
-    <row r="107" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>389</v>
+      </c>
+      <c r="S106" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="107" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
       <c r="B107" s="2" t="s">
         <v>300</v>
@@ -8493,19 +8508,19 @@
       <c r="D107" s="2"/>
       <c r="E107" s="2"/>
       <c r="F107" s="2" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="H107" s="2" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="I107" s="2" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="J107" s="8">
-        <v>4.4000000000000004</v>
+        <v>4</v>
       </c>
       <c r="K107" s="16">
         <v>250</v>
@@ -8529,13 +8544,11 @@
       <c r="R107" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="S107" s="2">
-        <v>1.9</v>
-      </c>
+      <c r="S107" s="2"/>
     </row>
     <row r="108" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
-        <v>903</v>
+        <v>396</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>300</v>
@@ -8546,19 +8559,19 @@
       <c r="D108" s="2"/>
       <c r="E108" s="2"/>
       <c r="F108" s="2" t="s">
-        <v>902</v>
+        <v>397</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>904</v>
+        <v>398</v>
       </c>
       <c r="H108" s="2" t="s">
-        <v>905</v>
+        <v>399</v>
       </c>
       <c r="I108" s="2" t="s">
-        <v>906</v>
+        <v>400</v>
       </c>
       <c r="J108" s="8">
-        <v>4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="K108" s="16">
         <v>250</v>
@@ -8582,11 +8595,13 @@
       <c r="R108" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="S108" s="2"/>
+      <c r="S108" s="2">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="109" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
-        <v>401</v>
+        <v>903</v>
       </c>
       <c r="B109" s="2" t="s">
         <v>300</v>
@@ -8597,19 +8612,19 @@
       <c r="D109" s="2"/>
       <c r="E109" s="2"/>
       <c r="F109" s="2" t="s">
-        <v>402</v>
+        <v>902</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>403</v>
+        <v>904</v>
       </c>
       <c r="H109" s="2" t="s">
-        <v>404</v>
+        <v>905</v>
       </c>
       <c r="I109" s="2" t="s">
-        <v>405</v>
+        <v>906</v>
       </c>
       <c r="J109" s="8">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="K109" s="16">
         <v>250</v>
@@ -8637,7 +8652,7 @@
     </row>
     <row r="110" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="B110" s="2" t="s">
         <v>300</v>
@@ -8648,22 +8663,22 @@
       <c r="D110" s="2"/>
       <c r="E110" s="2"/>
       <c r="F110" s="2" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
       <c r="I110" s="2" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
       <c r="J110" s="8">
-        <v>3.8</v>
+        <v>3.6</v>
       </c>
       <c r="K110" s="16">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="L110" s="2" t="s">
         <v>24</v>
@@ -8688,7 +8703,7 @@
     </row>
     <row r="111" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="B111" s="2" t="s">
         <v>300</v>
@@ -8699,16 +8714,16 @@
       <c r="D111" s="2"/>
       <c r="E111" s="2"/>
       <c r="F111" s="2" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>413</v>
+        <v>408</v>
       </c>
       <c r="H111" s="2" t="s">
-        <v>414</v>
+        <v>409</v>
       </c>
       <c r="I111" s="2" t="s">
-        <v>415</v>
+        <v>410</v>
       </c>
       <c r="J111" s="8">
         <v>3.8</v>
@@ -8739,7 +8754,7 @@
     </row>
     <row r="112" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
-        <v>416</v>
+        <v>411</v>
       </c>
       <c r="B112" s="2" t="s">
         <v>300</v>
@@ -8750,22 +8765,22 @@
       <c r="D112" s="2"/>
       <c r="E112" s="2"/>
       <c r="F112" s="2" t="s">
-        <v>417</v>
+        <v>412</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>418</v>
+        <v>413</v>
       </c>
       <c r="H112" s="2" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="I112" s="2" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
       <c r="J112" s="8">
         <v>3.8</v>
       </c>
       <c r="K112" s="16">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="L112" s="2" t="s">
         <v>24</v>
@@ -8788,9 +8803,9 @@
       </c>
       <c r="S112" s="2"/>
     </row>
-    <row r="113" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
-        <v>421</v>
+        <v>416</v>
       </c>
       <c r="B113" s="2" t="s">
         <v>300</v>
@@ -8801,16 +8816,16 @@
       <c r="D113" s="2"/>
       <c r="E113" s="2"/>
       <c r="F113" s="2" t="s">
-        <v>422</v>
+        <v>417</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>423</v>
+        <v>418</v>
       </c>
       <c r="H113" s="2" t="s">
-        <v>424</v>
+        <v>419</v>
       </c>
       <c r="I113" s="2" t="s">
-        <v>425</v>
+        <v>420</v>
       </c>
       <c r="J113" s="8">
         <v>3.8</v>
@@ -8839,9 +8854,9 @@
       </c>
       <c r="S113" s="2"/>
     </row>
-    <row r="114" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
-        <v>426</v>
+        <v>421</v>
       </c>
       <c r="B114" s="2" t="s">
         <v>300</v>
@@ -8852,19 +8867,19 @@
       <c r="D114" s="2"/>
       <c r="E114" s="2"/>
       <c r="F114" s="2" t="s">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="H114" s="2" t="s">
-        <v>429</v>
+        <v>424</v>
       </c>
       <c r="I114" s="2" t="s">
-        <v>430</v>
+        <v>425</v>
       </c>
       <c r="J114" s="8">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
       <c r="K114" s="16">
         <v>250</v>
@@ -8892,7 +8907,7 @@
     </row>
     <row r="115" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
-        <v>431</v>
+        <v>426</v>
       </c>
       <c r="B115" s="2" t="s">
         <v>300</v>
@@ -8903,19 +8918,19 @@
       <c r="D115" s="2"/>
       <c r="E115" s="2"/>
       <c r="F115" s="2" t="s">
-        <v>432</v>
+        <v>427</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>433</v>
+        <v>428</v>
       </c>
       <c r="H115" s="2" t="s">
-        <v>434</v>
+        <v>429</v>
       </c>
       <c r="I115" s="2" t="s">
-        <v>435</v>
+        <v>430</v>
       </c>
       <c r="J115" s="8">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K115" s="16">
         <v>250</v>
@@ -8941,9 +8956,9 @@
       </c>
       <c r="S115" s="2"/>
     </row>
-    <row r="116" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
-        <v>436</v>
+        <v>431</v>
       </c>
       <c r="B116" s="2" t="s">
         <v>300</v>
@@ -8954,29 +8969,27 @@
       <c r="D116" s="2"/>
       <c r="E116" s="2"/>
       <c r="F116" s="2" t="s">
-        <v>437</v>
+        <v>432</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>438</v>
+        <v>433</v>
       </c>
       <c r="H116" s="2" t="s">
-        <v>439</v>
+        <v>434</v>
       </c>
       <c r="I116" s="2" t="s">
-        <v>440</v>
+        <v>435</v>
       </c>
       <c r="J116" s="8">
         <v>4</v>
       </c>
       <c r="K116" s="16">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="L116" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M116" s="2" t="s">
-        <v>441</v>
-      </c>
+      <c r="M116" s="2"/>
       <c r="N116" s="2" t="b">
         <v>0</v>
       </c>
@@ -8994,9 +9007,9 @@
       </c>
       <c r="S116" s="2"/>
     </row>
-    <row r="117" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>300</v>
@@ -9007,16 +9020,16 @@
       <c r="D117" s="2"/>
       <c r="E117" s="2"/>
       <c r="F117" s="2" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
       <c r="H117" s="2" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="I117" s="2" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
       <c r="J117" s="8">
         <v>4</v>
@@ -9049,34 +9062,40 @@
     </row>
     <row r="118" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>43</v>
+        <v>300</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>292</v>
+        <v>384</v>
       </c>
       <c r="D118" s="2"/>
       <c r="E118" s="2"/>
       <c r="F118" s="2" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>450</v>
-      </c>
-      <c r="H118" s="2"/>
-      <c r="I118" s="2"/>
-      <c r="J118" s="18">
-        <v>3.8</v>
+        <v>444</v>
+      </c>
+      <c r="H118" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="I118" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="J118" s="8">
+        <v>4</v>
       </c>
       <c r="K118" s="16">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="L118" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M118" s="2"/>
+        <v>24</v>
+      </c>
+      <c r="M118" s="2" t="s">
+        <v>441</v>
+      </c>
       <c r="N118" s="2" t="b">
         <v>0</v>
       </c>
@@ -9090,39 +9109,35 @@
         <v>1</v>
       </c>
       <c r="R118" s="2" t="s">
-        <v>297</v>
+        <v>395</v>
       </c>
       <c r="S118" s="2"/>
     </row>
     <row r="119" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="B119" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>54</v>
+        <v>292</v>
       </c>
       <c r="D119" s="2"/>
       <c r="E119" s="2"/>
       <c r="F119" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>453</v>
-      </c>
-      <c r="H119" s="2" t="s">
-        <v>454</v>
-      </c>
-      <c r="I119" s="2" t="s">
-        <v>455</v>
-      </c>
-      <c r="J119" s="8">
-        <v>4.5</v>
+        <v>450</v>
+      </c>
+      <c r="H119" s="2"/>
+      <c r="I119" s="2"/>
+      <c r="J119" s="18">
+        <v>3.8</v>
       </c>
       <c r="K119" s="16">
-        <v>160</v>
+        <v>300</v>
       </c>
       <c r="L119" s="2" t="s">
         <v>57</v>
@@ -9141,44 +9156,42 @@
         <v>1</v>
       </c>
       <c r="R119" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="S119" s="2" t="s">
-        <v>375</v>
-      </c>
+        <v>297</v>
+      </c>
+      <c r="S119" s="2"/>
     </row>
     <row r="120" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
-        <v>456</v>
+        <v>451</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>300</v>
+        <v>43</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>384</v>
+        <v>54</v>
       </c>
       <c r="D120" s="2"/>
       <c r="E120" s="2"/>
       <c r="F120" s="2" t="s">
-        <v>457</v>
+        <v>452</v>
       </c>
       <c r="G120" s="2" t="s">
-        <v>458</v>
+        <v>453</v>
       </c>
       <c r="H120" s="2" t="s">
-        <v>459</v>
+        <v>454</v>
       </c>
       <c r="I120" s="2" t="s">
-        <v>460</v>
-      </c>
-      <c r="J120" s="10">
-        <v>4</v>
+        <v>455</v>
+      </c>
+      <c r="J120" s="8">
+        <v>4.5</v>
       </c>
       <c r="K120" s="16">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="L120" s="2" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="M120" s="2"/>
       <c r="N120" s="2" t="b">
@@ -9194,46 +9207,46 @@
         <v>1</v>
       </c>
       <c r="R120" s="2" t="s">
-        <v>395</v>
-      </c>
-      <c r="S120" s="2"/>
-    </row>
-    <row r="121" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="S120" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="121" spans="1:19" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
-        <v>461</v>
+        <v>456</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>43</v>
+        <v>300</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>54</v>
+        <v>384</v>
       </c>
       <c r="D121" s="2"/>
       <c r="E121" s="2"/>
       <c r="F121" s="2" t="s">
-        <v>462</v>
+        <v>457</v>
       </c>
       <c r="G121" s="2" t="s">
-        <v>463</v>
+        <v>458</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>464</v>
+        <v>459</v>
       </c>
       <c r="I121" s="2" t="s">
-        <v>465</v>
+        <v>460</v>
       </c>
       <c r="J121" s="10">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="K121" s="16">
-        <v>270</v>
+        <v>200</v>
       </c>
       <c r="L121" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M121" s="2" t="s">
-        <v>466</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="M121" s="2"/>
       <c r="N121" s="2" t="b">
         <v>0</v>
       </c>
@@ -9247,42 +9260,46 @@
         <v>1</v>
       </c>
       <c r="R121" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="S121" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="122" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>395</v>
+      </c>
+      <c r="S121" s="2"/>
+    </row>
+    <row r="122" spans="1:19" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
-        <v>467</v>
+        <v>461</v>
       </c>
       <c r="B122" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>292</v>
+        <v>54</v>
       </c>
       <c r="D122" s="2"/>
       <c r="E122" s="2"/>
       <c r="F122" s="2" t="s">
-        <v>468</v>
+        <v>462</v>
       </c>
       <c r="G122" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="H122" s="2"/>
-      <c r="I122" s="2"/>
-      <c r="J122" s="18">
-        <v>4</v>
+        <v>463</v>
+      </c>
+      <c r="H122" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="I122" s="2" t="s">
+        <v>465</v>
+      </c>
+      <c r="J122" s="10">
+        <v>3.9</v>
       </c>
       <c r="K122" s="16">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="L122" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M122" s="2"/>
+      <c r="M122" s="2" t="s">
+        <v>466</v>
+      </c>
       <c r="N122" s="2" t="b">
         <v>0</v>
       </c>
@@ -9296,46 +9313,42 @@
         <v>1</v>
       </c>
       <c r="R122" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S122" s="2"/>
-    </row>
-    <row r="123" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+      <c r="S122" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="123" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>300</v>
+        <v>43</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>384</v>
+        <v>292</v>
       </c>
       <c r="D123" s="2"/>
       <c r="E123" s="2"/>
       <c r="F123" s="2" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="G123" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="H123" s="2" t="s">
-        <v>473</v>
-      </c>
-      <c r="I123" s="2" t="s">
-        <v>474</v>
-      </c>
-      <c r="J123" s="8">
-        <v>4.4000000000000004</v>
+        <v>469</v>
+      </c>
+      <c r="H123" s="2"/>
+      <c r="I123" s="2"/>
+      <c r="J123" s="18">
+        <v>4</v>
       </c>
       <c r="K123" s="16">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="L123" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M123" s="2" t="s">
-        <v>831</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="M123" s="2"/>
       <c r="N123" s="2" t="b">
         <v>0</v>
       </c>
@@ -9349,13 +9362,13 @@
         <v>1</v>
       </c>
       <c r="R123" s="2" t="s">
-        <v>395</v>
+        <v>297</v>
       </c>
       <c r="S123" s="2"/>
     </row>
     <row r="124" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
-        <v>475</v>
+        <v>470</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>300</v>
@@ -9366,27 +9379,29 @@
       <c r="D124" s="2"/>
       <c r="E124" s="2"/>
       <c r="F124" s="2" t="s">
-        <v>476</v>
+        <v>471</v>
       </c>
       <c r="G124" s="2" t="s">
-        <v>477</v>
+        <v>472</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>478</v>
+        <v>473</v>
       </c>
       <c r="I124" s="2" t="s">
-        <v>479</v>
+        <v>474</v>
       </c>
       <c r="J124" s="8">
         <v>4.4000000000000004</v>
       </c>
       <c r="K124" s="16">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="L124" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M124" s="2"/>
+      <c r="M124" s="2" t="s">
+        <v>831</v>
+      </c>
       <c r="N124" s="2" t="b">
         <v>0</v>
       </c>
@@ -9404,9 +9419,9 @@
       </c>
       <c r="S124" s="2"/>
     </row>
-    <row r="125" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
-        <v>480</v>
+        <v>475</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>300</v>
@@ -9417,22 +9432,22 @@
       <c r="D125" s="2"/>
       <c r="E125" s="2"/>
       <c r="F125" s="2" t="s">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="G125" s="2" t="s">
-        <v>482</v>
+        <v>477</v>
       </c>
       <c r="H125" s="2" t="s">
-        <v>483</v>
+        <v>478</v>
       </c>
       <c r="I125" s="2" t="s">
-        <v>484</v>
+        <v>479</v>
       </c>
       <c r="J125" s="8">
-        <v>4</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="K125" s="16">
-        <v>150</v>
+        <v>250</v>
       </c>
       <c r="L125" s="2" t="s">
         <v>24</v>
@@ -9455,9 +9470,9 @@
       </c>
       <c r="S125" s="2"/>
     </row>
-    <row r="126" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
-        <v>485</v>
+        <v>480</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>300</v>
@@ -9468,29 +9483,27 @@
       <c r="D126" s="2"/>
       <c r="E126" s="2"/>
       <c r="F126" s="2" t="s">
-        <v>486</v>
+        <v>481</v>
       </c>
       <c r="G126" s="2" t="s">
-        <v>487</v>
+        <v>482</v>
       </c>
       <c r="H126" s="2" t="s">
-        <v>488</v>
+        <v>483</v>
       </c>
       <c r="I126" s="2" t="s">
-        <v>489</v>
+        <v>484</v>
       </c>
       <c r="J126" s="8">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="K126" s="16">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="L126" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M126" s="2" t="s">
-        <v>830</v>
-      </c>
+      <c r="M126" s="2"/>
       <c r="N126" s="2" t="b">
         <v>0</v>
       </c>
@@ -9508,9 +9521,9 @@
       </c>
       <c r="S126" s="2"/>
     </row>
-    <row r="127" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
-        <v>490</v>
+        <v>485</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>300</v>
@@ -9521,19 +9534,19 @@
       <c r="D127" s="2"/>
       <c r="E127" s="2"/>
       <c r="F127" s="2" t="s">
-        <v>491</v>
+        <v>486</v>
       </c>
       <c r="G127" s="2" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="H127" s="2" t="s">
-        <v>493</v>
+        <v>488</v>
       </c>
       <c r="I127" s="2" t="s">
-        <v>494</v>
+        <v>489</v>
       </c>
       <c r="J127" s="8">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K127" s="16">
         <v>250</v>
@@ -9541,7 +9554,9 @@
       <c r="L127" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M127" s="2"/>
+      <c r="M127" s="2" t="s">
+        <v>830</v>
+      </c>
       <c r="N127" s="2" t="b">
         <v>0</v>
       </c>
@@ -9559,9 +9574,9 @@
       </c>
       <c r="S127" s="2"/>
     </row>
-    <row r="128" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
-        <v>495</v>
+        <v>490</v>
       </c>
       <c r="B128" s="2" t="s">
         <v>300</v>
@@ -9572,19 +9587,19 @@
       <c r="D128" s="2"/>
       <c r="E128" s="2"/>
       <c r="F128" s="2" t="s">
-        <v>496</v>
+        <v>491</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>497</v>
+        <v>492</v>
       </c>
       <c r="H128" s="2" t="s">
-        <v>498</v>
+        <v>493</v>
       </c>
       <c r="I128" s="2" t="s">
-        <v>499</v>
+        <v>494</v>
       </c>
       <c r="J128" s="8">
-        <v>4.4000000000000004</v>
+        <v>4</v>
       </c>
       <c r="K128" s="16">
         <v>250</v>
@@ -9610,9 +9625,9 @@
       </c>
       <c r="S128" s="2"/>
     </row>
-    <row r="129" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="B129" s="2" t="s">
         <v>300</v>
@@ -9623,16 +9638,16 @@
       <c r="D129" s="2"/>
       <c r="E129" s="2"/>
       <c r="F129" s="2" t="s">
-        <v>501</v>
+        <v>496</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>502</v>
+        <v>497</v>
       </c>
       <c r="H129" s="2" t="s">
-        <v>503</v>
+        <v>498</v>
       </c>
       <c r="I129" s="2" t="s">
-        <v>504</v>
+        <v>499</v>
       </c>
       <c r="J129" s="8">
         <v>4.4000000000000004</v>
@@ -9661,9 +9676,9 @@
       </c>
       <c r="S129" s="2"/>
     </row>
-    <row r="130" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
-        <v>505</v>
+        <v>500</v>
       </c>
       <c r="B130" s="2" t="s">
         <v>300</v>
@@ -9674,19 +9689,19 @@
       <c r="D130" s="2"/>
       <c r="E130" s="2"/>
       <c r="F130" s="2" t="s">
-        <v>506</v>
+        <v>501</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>507</v>
+        <v>502</v>
       </c>
       <c r="H130" s="2" t="s">
-        <v>508</v>
+        <v>503</v>
       </c>
       <c r="I130" s="2" t="s">
-        <v>509</v>
+        <v>504</v>
       </c>
       <c r="J130" s="8">
-        <v>4.5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="K130" s="16">
         <v>250</v>
@@ -9694,9 +9709,7 @@
       <c r="L130" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M130" s="2" t="s">
-        <v>835</v>
-      </c>
+      <c r="M130" s="2"/>
       <c r="N130" s="2" t="b">
         <v>0</v>
       </c>
@@ -9714,9 +9727,9 @@
       </c>
       <c r="S130" s="2"/>
     </row>
-    <row r="131" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
-        <v>510</v>
+        <v>505</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>300</v>
@@ -9727,27 +9740,29 @@
       <c r="D131" s="2"/>
       <c r="E131" s="2"/>
       <c r="F131" s="2" t="s">
-        <v>511</v>
+        <v>506</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>512</v>
+        <v>507</v>
       </c>
       <c r="H131" s="2" t="s">
-        <v>513</v>
+        <v>508</v>
       </c>
       <c r="I131" s="2" t="s">
-        <v>514</v>
+        <v>509</v>
       </c>
       <c r="J131" s="8">
-        <v>4.4000000000000004</v>
+        <v>4.5</v>
       </c>
       <c r="K131" s="16">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="L131" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="M131" s="2"/>
+      <c r="M131" s="2" t="s">
+        <v>835</v>
+      </c>
       <c r="N131" s="2" t="b">
         <v>0</v>
       </c>
@@ -9763,13 +9778,11 @@
       <c r="R131" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="S131" s="2">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="132" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S131" s="2"/>
+    </row>
+    <row r="132" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
-        <v>515</v>
+        <v>510</v>
       </c>
       <c r="B132" s="2" t="s">
         <v>300</v>
@@ -9780,21 +9793,23 @@
       <c r="D132" s="2"/>
       <c r="E132" s="2"/>
       <c r="F132" s="2" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="H132" s="2" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
       <c r="I132" s="2" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
       <c r="J132" s="8">
         <v>4.4000000000000004</v>
       </c>
-      <c r="K132" s="16"/>
+      <c r="K132" s="16">
+        <v>200</v>
+      </c>
       <c r="L132" s="2" t="s">
         <v>24</v>
       </c>
@@ -9818,86 +9833,90 @@
         <v>7</v>
       </c>
     </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A133" t="s">
+    <row r="133" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="B133" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C133" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="D133" s="2"/>
+      <c r="E133" s="2"/>
+      <c r="F133" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="G133" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="H133" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="I133" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="J133" s="8">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="K133" s="16"/>
+      <c r="L133" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M133" s="2"/>
+      <c r="N133" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O133" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P133" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q133" t="b">
+        <v>1</v>
+      </c>
+      <c r="R133" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="S133" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="134" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
         <v>520</v>
-      </c>
-      <c r="B133" t="s">
-        <v>20</v>
-      </c>
-      <c r="C133" t="s">
-        <v>266</v>
-      </c>
-      <c r="D133" t="s">
-        <v>521</v>
-      </c>
-      <c r="E133" t="s">
-        <v>522</v>
-      </c>
-      <c r="F133" t="s">
-        <v>847</v>
-      </c>
-      <c r="G133" t="s">
-        <v>523</v>
-      </c>
-      <c r="J133" s="9">
-        <v>2.4</v>
-      </c>
-      <c r="K133" s="15">
-        <v>330</v>
-      </c>
-      <c r="L133" t="s">
-        <v>24</v>
-      </c>
-      <c r="N133" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="O133" t="b">
-        <v>0</v>
-      </c>
-      <c r="P133" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q133" t="b">
-        <v>1</v>
-      </c>
-      <c r="R133" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="134" spans="1:19" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A134" t="s">
-        <v>525</v>
       </c>
       <c r="B134" t="s">
         <v>20</v>
       </c>
       <c r="C134" t="s">
-        <v>526</v>
+        <v>266</v>
       </c>
       <c r="D134" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
       <c r="E134" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="F134" t="s">
-        <v>529</v>
+        <v>847</v>
       </c>
       <c r="G134" t="s">
-        <v>530</v>
+        <v>523</v>
       </c>
       <c r="J134" s="9">
-        <v>3.7</v>
+        <v>2.4</v>
       </c>
       <c r="K134" s="15">
-        <v>200</v>
+        <v>330</v>
       </c>
       <c r="L134" t="s">
         <v>24</v>
       </c>
       <c r="N134" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O134" t="b">
         <v>0</v>
@@ -9912,9 +9931,9 @@
         <v>524</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:19" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
-        <v>531</v>
+        <v>525</v>
       </c>
       <c r="B135" t="s">
         <v>20</v>
@@ -9926,13 +9945,13 @@
         <v>527</v>
       </c>
       <c r="E135" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="F135" t="s">
-        <v>533</v>
+        <v>529</v>
       </c>
       <c r="G135" t="s">
-        <v>534</v>
+        <v>530</v>
       </c>
       <c r="J135" s="9">
         <v>3.7</v>
@@ -9961,7 +9980,7 @@
     </row>
     <row r="136" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
-        <v>535</v>
+        <v>531</v>
       </c>
       <c r="B136" t="s">
         <v>20</v>
@@ -9973,13 +9992,13 @@
         <v>527</v>
       </c>
       <c r="E136" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="F136" t="s">
-        <v>537</v>
+        <v>533</v>
       </c>
       <c r="G136" t="s">
-        <v>538</v>
+        <v>534</v>
       </c>
       <c r="J136" s="9">
         <v>3.7</v>
@@ -10006,39 +10025,33 @@
         <v>524</v>
       </c>
     </row>
-    <row r="137" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
-        <v>539</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>300</v>
+        <v>535</v>
+      </c>
+      <c r="B137" t="s">
+        <v>20</v>
       </c>
       <c r="C137" t="s">
-        <v>540</v>
+        <v>526</v>
       </c>
       <c r="D137" t="s">
-        <v>282</v>
+        <v>527</v>
       </c>
       <c r="E137" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F137" t="s">
-        <v>541</v>
+        <v>537</v>
       </c>
       <c r="G137" t="s">
-        <v>542</v>
-      </c>
-      <c r="H137" t="s">
-        <v>543</v>
-      </c>
-      <c r="I137" t="s">
-        <v>544</v>
+        <v>538</v>
       </c>
       <c r="J137" s="9">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="K137" s="15">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="L137" t="s">
         <v>24</v>
@@ -10056,12 +10069,12 @@
         <v>1</v>
       </c>
       <c r="R137" t="s">
-        <v>545</v>
+        <v>524</v>
       </c>
     </row>
     <row r="138" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
       <c r="B138" s="2" t="s">
         <v>300</v>
@@ -10073,25 +10086,25 @@
         <v>282</v>
       </c>
       <c r="E138" t="s">
-        <v>546</v>
+        <v>539</v>
       </c>
       <c r="F138" t="s">
-        <v>547</v>
+        <v>541</v>
       </c>
       <c r="G138" t="s">
-        <v>548</v>
+        <v>542</v>
       </c>
       <c r="H138" t="s">
-        <v>549</v>
+        <v>543</v>
       </c>
       <c r="I138" t="s">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="J138" s="9">
         <v>3.6</v>
       </c>
       <c r="K138" s="15">
-        <v>200</v>
+        <v>250</v>
       </c>
       <c r="L138" t="s">
         <v>24</v>
@@ -10114,7 +10127,7 @@
     </row>
     <row r="139" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
-        <v>551</v>
+        <v>546</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>300</v>
@@ -10126,25 +10139,25 @@
         <v>282</v>
       </c>
       <c r="E139" t="s">
-        <v>470</v>
+        <v>546</v>
       </c>
       <c r="F139" t="s">
-        <v>471</v>
+        <v>547</v>
       </c>
       <c r="G139" t="s">
-        <v>552</v>
+        <v>548</v>
       </c>
       <c r="H139" t="s">
-        <v>553</v>
+        <v>549</v>
       </c>
       <c r="I139" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
       <c r="J139" s="9">
         <v>3.6</v>
       </c>
       <c r="K139" s="15">
-        <v>250</v>
+        <v>200</v>
       </c>
       <c r="L139" t="s">
         <v>24</v>
@@ -10167,7 +10180,7 @@
     </row>
     <row r="140" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
-        <v>555</v>
+        <v>551</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>300</v>
@@ -10179,22 +10192,22 @@
         <v>282</v>
       </c>
       <c r="E140" t="s">
-        <v>555</v>
+        <v>470</v>
       </c>
       <c r="F140" t="s">
-        <v>556</v>
+        <v>471</v>
       </c>
       <c r="G140" t="s">
-        <v>557</v>
+        <v>552</v>
       </c>
       <c r="H140" t="s">
-        <v>558</v>
+        <v>553</v>
       </c>
       <c r="I140" t="s">
-        <v>559</v>
+        <v>554</v>
       </c>
       <c r="J140" s="9">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="K140" s="15">
         <v>250</v>
@@ -10220,7 +10233,7 @@
     </row>
     <row r="141" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>300</v>
@@ -10232,25 +10245,25 @@
         <v>282</v>
       </c>
       <c r="E141" t="s">
-        <v>560</v>
+        <v>555</v>
       </c>
       <c r="F141" t="s">
-        <v>561</v>
+        <v>556</v>
       </c>
       <c r="G141" t="s">
-        <v>562</v>
+        <v>557</v>
       </c>
       <c r="H141" t="s">
-        <v>563</v>
+        <v>558</v>
       </c>
       <c r="I141" t="s">
-        <v>564</v>
+        <v>559</v>
       </c>
       <c r="J141" s="9">
         <v>4</v>
       </c>
       <c r="K141" s="15">
-        <v>330</v>
+        <v>250</v>
       </c>
       <c r="L141" t="s">
         <v>24</v>
@@ -10273,7 +10286,7 @@
     </row>
     <row r="142" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>300</v>
@@ -10285,22 +10298,22 @@
         <v>282</v>
       </c>
       <c r="E142" t="s">
-        <v>565</v>
+        <v>560</v>
       </c>
       <c r="F142" t="s">
-        <v>566</v>
+        <v>561</v>
       </c>
       <c r="G142" t="s">
-        <v>567</v>
+        <v>562</v>
       </c>
       <c r="H142" t="s">
-        <v>568</v>
+        <v>563</v>
       </c>
       <c r="I142" t="s">
-        <v>569</v>
+        <v>564</v>
       </c>
       <c r="J142" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K142" s="15">
         <v>330</v>
@@ -10321,12 +10334,12 @@
         <v>1</v>
       </c>
       <c r="R142" t="s">
-        <v>570</v>
+        <v>545</v>
       </c>
     </row>
     <row r="143" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="B143" s="2" t="s">
         <v>300</v>
@@ -10338,22 +10351,22 @@
         <v>282</v>
       </c>
       <c r="E143" t="s">
-        <v>571</v>
+        <v>565</v>
       </c>
       <c r="F143" t="s">
-        <v>572</v>
+        <v>566</v>
       </c>
       <c r="G143" t="s">
-        <v>573</v>
+        <v>567</v>
       </c>
       <c r="H143" t="s">
-        <v>574</v>
+        <v>568</v>
       </c>
       <c r="I143" t="s">
-        <v>575</v>
+        <v>569</v>
       </c>
       <c r="J143" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K143" s="15">
         <v>330</v>
@@ -10377,58 +10390,62 @@
         <v>570</v>
       </c>
     </row>
-    <row r="144" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A144" s="2" t="s">
+    <row r="144" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>571</v>
+      </c>
+      <c r="B144" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C144" t="s">
+        <v>540</v>
+      </c>
+      <c r="D144" t="s">
+        <v>282</v>
+      </c>
+      <c r="E144" t="s">
+        <v>571</v>
+      </c>
+      <c r="F144" t="s">
+        <v>572</v>
+      </c>
+      <c r="G144" t="s">
+        <v>573</v>
+      </c>
+      <c r="H144" t="s">
+        <v>574</v>
+      </c>
+      <c r="I144" t="s">
+        <v>575</v>
+      </c>
+      <c r="J144" s="9">
+        <v>4</v>
+      </c>
+      <c r="K144" s="15">
+        <v>330</v>
+      </c>
+      <c r="L144" t="s">
+        <v>24</v>
+      </c>
+      <c r="N144" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O144" t="b">
+        <v>0</v>
+      </c>
+      <c r="P144" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q144" t="b">
+        <v>1</v>
+      </c>
+      <c r="R144" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="145" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A145" s="2" t="s">
         <v>576</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
-      <c r="F144" s="2" t="s">
-        <v>577</v>
-      </c>
-      <c r="G144" s="2" t="s">
-        <v>578</v>
-      </c>
-      <c r="H144" s="2"/>
-      <c r="I144" s="2"/>
-      <c r="J144" s="18">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="K144" s="16">
-        <v>350</v>
-      </c>
-      <c r="L144" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M144" s="2" t="s">
-        <v>832</v>
-      </c>
-      <c r="N144" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O144" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P144" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q144" t="b">
-        <v>1</v>
-      </c>
-      <c r="R144" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S144" s="2"/>
-    </row>
-    <row r="145" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A145" s="2" t="s">
-        <v>579</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>43</v>
@@ -10439,28 +10456,24 @@
       <c r="D145" s="2"/>
       <c r="E145" s="2"/>
       <c r="F145" s="2" t="s">
-        <v>580</v>
+        <v>577</v>
       </c>
       <c r="G145" s="2" t="s">
-        <v>581</v>
-      </c>
-      <c r="H145" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="I145" s="2" t="s">
-        <v>583</v>
-      </c>
+        <v>578</v>
+      </c>
+      <c r="H145" s="2"/>
+      <c r="I145" s="2"/>
       <c r="J145" s="18">
-        <v>4.5</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="K145" s="16">
-        <v>260</v>
+        <v>350</v>
       </c>
       <c r="L145" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M145" s="2" t="s">
-        <v>834</v>
+        <v>832</v>
       </c>
       <c r="N145" s="2" t="b">
         <v>0</v>
@@ -10477,44 +10490,44 @@
       <c r="R145" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="S145" s="2" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="146" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S145" s="2"/>
+    </row>
+    <row r="146" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
-        <v>584</v>
+        <v>579</v>
       </c>
       <c r="B146" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>54</v>
+        <v>292</v>
       </c>
       <c r="D146" s="2"/>
       <c r="E146" s="2"/>
       <c r="F146" s="2" t="s">
-        <v>585</v>
+        <v>580</v>
       </c>
       <c r="G146" s="2" t="s">
-        <v>586</v>
+        <v>581</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>587</v>
+        <v>582</v>
       </c>
       <c r="I146" s="2" t="s">
-        <v>588</v>
-      </c>
-      <c r="J146" s="8">
-        <v>4.0999999999999996</v>
+        <v>583</v>
+      </c>
+      <c r="J146" s="18">
+        <v>4.5</v>
       </c>
       <c r="K146" s="16">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="L146" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M146" s="2"/>
+      <c r="M146" s="2" t="s">
+        <v>834</v>
+      </c>
       <c r="N146" s="2" t="b">
         <v>0</v>
       </c>
@@ -10528,145 +10541,147 @@
         <v>1</v>
       </c>
       <c r="R146" s="2" t="s">
-        <v>58</v>
+        <v>297</v>
       </c>
       <c r="S146" s="2" t="s">
-        <v>375</v>
-      </c>
-    </row>
-    <row r="147" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="147" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
-        <v>589</v>
+        <v>584</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>300</v>
+        <v>43</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>384</v>
+        <v>54</v>
       </c>
       <c r="D147" s="2"/>
       <c r="E147" s="2"/>
       <c r="F147" s="2" t="s">
+        <v>585</v>
+      </c>
+      <c r="G147" s="2" t="s">
+        <v>586</v>
+      </c>
+      <c r="H147" s="2" t="s">
+        <v>587</v>
+      </c>
+      <c r="I147" s="2" t="s">
+        <v>588</v>
+      </c>
+      <c r="J147" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="K147" s="16">
+        <v>270</v>
+      </c>
+      <c r="L147" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M147" s="2"/>
+      <c r="N147" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O147" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P147" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q147" t="b">
+        <v>1</v>
+      </c>
+      <c r="R147" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="S147" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="148" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A148" s="2" t="s">
+        <v>589</v>
+      </c>
+      <c r="B148" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="D148" s="2"/>
+      <c r="E148" s="2"/>
+      <c r="F148" s="2" t="s">
         <v>590</v>
       </c>
-      <c r="G147" s="2" t="s">
+      <c r="G148" s="2" t="s">
         <v>591</v>
       </c>
-      <c r="H147" s="2" t="s">
+      <c r="H148" s="2" t="s">
         <v>592</v>
       </c>
-      <c r="I147" s="2" t="s">
+      <c r="I148" s="2" t="s">
         <v>593</v>
       </c>
-      <c r="J147" s="8">
+      <c r="J148" s="8">
         <v>4.2</v>
       </c>
-      <c r="K147" s="16">
+      <c r="K148" s="16">
         <v>250</v>
       </c>
-      <c r="L147" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M147" s="2" t="s">
+      <c r="L148" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M148" s="2" t="s">
         <v>594</v>
       </c>
-      <c r="N147" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O147" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P147" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q147" t="b">
-        <v>1</v>
-      </c>
-      <c r="R147" s="2" t="s">
+      <c r="N148" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O148" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P148" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q148" t="b">
+        <v>1</v>
+      </c>
+      <c r="R148" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="S147" s="2"/>
-    </row>
-    <row r="148" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A148" s="2" t="s">
+      <c r="S148" s="2"/>
+    </row>
+    <row r="149" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A149" s="2" t="s">
         <v>596</v>
       </c>
-      <c r="B148" s="2" t="s">
+      <c r="B149" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C148" s="2" t="s">
+      <c r="C149" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D148" s="2" t="s">
+      <c r="D149" s="2" t="s">
         <v>597</v>
       </c>
-      <c r="E148" s="2" t="s">
+      <c r="E149" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="F148" s="2" t="s">
+      <c r="F149" s="2" t="s">
         <v>882</v>
       </c>
-      <c r="G148" s="2" t="s">
+      <c r="G149" s="2" t="s">
         <v>883</v>
       </c>
-      <c r="H148" s="2"/>
-      <c r="I148" s="2"/>
-      <c r="J148" s="8">
+      <c r="H149" s="2"/>
+      <c r="I149" s="2"/>
+      <c r="J149" s="8">
         <v>4.5</v>
       </c>
-      <c r="K148" s="16">
+      <c r="K149" s="16">
         <v>50</v>
-      </c>
-      <c r="L148" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M148" s="2"/>
-      <c r="N148" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O148" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P148" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q148" t="b">
-        <v>1</v>
-      </c>
-      <c r="R148" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="S148" s="2"/>
-    </row>
-    <row r="149" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A149" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C149" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D149" s="2"/>
-      <c r="E149" s="2"/>
-      <c r="F149" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="G149" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="H149" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="I149" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="J149" s="8">
-        <v>4.4000000000000004</v>
-      </c>
-      <c r="K149" s="16">
-        <v>300</v>
       </c>
       <c r="L149" s="2" t="s">
         <v>24</v>
@@ -10685,13 +10700,13 @@
         <v>1</v>
       </c>
       <c r="R149" s="2" t="s">
-        <v>595</v>
+        <v>68</v>
       </c>
       <c r="S149" s="2"/>
     </row>
-    <row r="150" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:19" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
-        <v>603</v>
+        <v>598</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>300</v>
@@ -10702,16 +10717,16 @@
       <c r="D150" s="2"/>
       <c r="E150" s="2"/>
       <c r="F150" s="2" t="s">
-        <v>604</v>
+        <v>599</v>
       </c>
       <c r="G150" s="2" t="s">
-        <v>605</v>
+        <v>600</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>606</v>
+        <v>601</v>
       </c>
       <c r="I150" s="2" t="s">
-        <v>607</v>
+        <v>602</v>
       </c>
       <c r="J150" s="8">
         <v>4.4000000000000004</v>
@@ -10740,9 +10755,9 @@
       </c>
       <c r="S150" s="2"/>
     </row>
-    <row r="151" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
-        <v>608</v>
+        <v>603</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>300</v>
@@ -10753,19 +10768,19 @@
       <c r="D151" s="2"/>
       <c r="E151" s="2"/>
       <c r="F151" s="2" t="s">
-        <v>609</v>
+        <v>604</v>
       </c>
       <c r="G151" s="2" t="s">
-        <v>610</v>
+        <v>605</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>611</v>
+        <v>606</v>
       </c>
       <c r="I151" s="2" t="s">
-        <v>612</v>
+        <v>607</v>
       </c>
       <c r="J151" s="8">
-        <v>5</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="K151" s="16">
         <v>300</v>
@@ -10791,9 +10806,9 @@
       </c>
       <c r="S151" s="2"/>
     </row>
-    <row r="152" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
-        <v>613</v>
+        <v>608</v>
       </c>
       <c r="B152" s="2" t="s">
         <v>300</v>
@@ -10804,19 +10819,19 @@
       <c r="D152" s="2"/>
       <c r="E152" s="2"/>
       <c r="F152" s="2" t="s">
-        <v>614</v>
+        <v>609</v>
       </c>
       <c r="G152" s="2" t="s">
-        <v>615</v>
+        <v>610</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>616</v>
+        <v>611</v>
       </c>
       <c r="I152" s="2" t="s">
-        <v>617</v>
+        <v>612</v>
       </c>
       <c r="J152" s="8">
-        <v>4.5999999999999996</v>
+        <v>5</v>
       </c>
       <c r="K152" s="16">
         <v>300</v>
@@ -10842,38 +10857,38 @@
       </c>
       <c r="S152" s="2"/>
     </row>
-    <row r="153" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
-        <v>618</v>
+        <v>613</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>43</v>
+        <v>300</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>619</v>
+        <v>37</v>
       </c>
       <c r="D153" s="2"/>
       <c r="E153" s="2"/>
       <c r="F153" s="2" t="s">
-        <v>620</v>
+        <v>614</v>
       </c>
       <c r="G153" s="2" t="s">
-        <v>621</v>
+        <v>615</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>622</v>
+        <v>616</v>
       </c>
       <c r="I153" s="2" t="s">
-        <v>623</v>
+        <v>617</v>
       </c>
       <c r="J153" s="8">
-        <v>5.4</v>
+        <v>4.5999999999999996</v>
       </c>
       <c r="K153" s="16">
         <v>300</v>
       </c>
       <c r="L153" s="2" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="M153" s="2"/>
       <c r="N153" s="2" t="b">
@@ -10889,44 +10904,42 @@
         <v>1</v>
       </c>
       <c r="R153" s="2" t="s">
-        <v>624</v>
-      </c>
-      <c r="S153" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="154" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>595</v>
+      </c>
+      <c r="S153" s="2"/>
+    </row>
+    <row r="154" spans="1:19" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
-        <v>625</v>
+        <v>618</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C154" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D154" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="E154" s="2" t="s">
-        <v>90</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="D154" s="2"/>
+      <c r="E154" s="2"/>
       <c r="F154" s="2" t="s">
-        <v>885</v>
+        <v>620</v>
       </c>
       <c r="G154" s="2" t="s">
-        <v>627</v>
-      </c>
-      <c r="H154" s="2"/>
-      <c r="I154" s="2"/>
-      <c r="J154" s="18">
-        <v>5</v>
+        <v>621</v>
+      </c>
+      <c r="H154" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="I154" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="J154" s="8">
+        <v>5.4</v>
       </c>
       <c r="K154" s="16">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="L154" s="2" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="M154" s="2"/>
       <c r="N154" s="2" t="b">
@@ -10942,27 +10955,33 @@
         <v>1</v>
       </c>
       <c r="R154" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="S154" s="2"/>
-    </row>
-    <row r="155" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>624</v>
+      </c>
+      <c r="S154" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="155" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
-        <v>629</v>
+        <v>625</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C155" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D155" s="2"/>
-      <c r="E155" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="C155" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D155" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="E155" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="F155" s="2" t="s">
-        <v>630</v>
+        <v>885</v>
       </c>
       <c r="G155" s="2" t="s">
-        <v>631</v>
+        <v>627</v>
       </c>
       <c r="H155" s="2"/>
       <c r="I155" s="2"/>
@@ -10970,10 +10989,10 @@
         <v>5</v>
       </c>
       <c r="K155" s="16">
-        <v>230</v>
+        <v>50</v>
       </c>
       <c r="L155" s="2" t="s">
-        <v>57</v>
+        <v>24</v>
       </c>
       <c r="M155" s="2"/>
       <c r="N155" s="2" t="b">
@@ -10989,41 +11008,35 @@
         <v>1</v>
       </c>
       <c r="R155" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S155" s="2">
-        <v>3.7</v>
-      </c>
-    </row>
-    <row r="156" spans="1:19" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+      <c r="S155" s="2"/>
+    </row>
+    <row r="156" spans="1:19" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
-        <v>632</v>
+        <v>629</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>619</v>
+        <v>292</v>
       </c>
       <c r="D156" s="2"/>
       <c r="E156" s="2"/>
       <c r="F156" s="2" t="s">
-        <v>633</v>
+        <v>630</v>
       </c>
       <c r="G156" s="2" t="s">
-        <v>634</v>
-      </c>
-      <c r="H156" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="I156" s="2" t="s">
-        <v>636</v>
-      </c>
-      <c r="J156" s="8">
-        <v>6.5</v>
+        <v>631</v>
+      </c>
+      <c r="H156" s="2"/>
+      <c r="I156" s="2"/>
+      <c r="J156" s="18">
+        <v>5</v>
       </c>
       <c r="K156" s="16">
-        <v>280</v>
+        <v>230</v>
       </c>
       <c r="L156" s="2" t="s">
         <v>57</v>
@@ -11042,68 +11055,68 @@
         <v>1</v>
       </c>
       <c r="R156" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="S156" s="2">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="157" spans="1:19" ht="151.80000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A157" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="B157" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="D157" s="2"/>
+      <c r="E157" s="2"/>
+      <c r="F157" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="G157" s="2" t="s">
+        <v>634</v>
+      </c>
+      <c r="H157" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="I157" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="J157" s="8">
+        <v>6.5</v>
+      </c>
+      <c r="K157" s="16">
+        <v>280</v>
+      </c>
+      <c r="L157" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M157" s="2"/>
+      <c r="N157" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O157" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P157" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q157" t="b">
+        <v>1</v>
+      </c>
+      <c r="R157" s="2" t="s">
         <v>624</v>
       </c>
-      <c r="S156" s="2" t="s">
+      <c r="S157" s="2" t="s">
         <v>447</v>
-      </c>
-    </row>
-    <row r="157" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>637</v>
-      </c>
-      <c r="B157" s="2" t="s">
-        <v>300</v>
-      </c>
-      <c r="C157" t="s">
-        <v>540</v>
-      </c>
-      <c r="D157" t="s">
-        <v>282</v>
-      </c>
-      <c r="E157" t="s">
-        <v>637</v>
-      </c>
-      <c r="F157" t="s">
-        <v>638</v>
-      </c>
-      <c r="G157" t="s">
-        <v>639</v>
-      </c>
-      <c r="H157" t="s">
-        <v>640</v>
-      </c>
-      <c r="I157" t="s">
-        <v>641</v>
-      </c>
-      <c r="J157" s="9">
-        <v>3.8</v>
-      </c>
-      <c r="K157" s="15">
-        <v>200</v>
-      </c>
-      <c r="L157" t="s">
-        <v>24</v>
-      </c>
-      <c r="N157" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O157" t="b">
-        <v>0</v>
-      </c>
-      <c r="P157" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q157" t="b">
-        <v>1</v>
-      </c>
-      <c r="R157" t="s">
-        <v>545</v>
       </c>
     </row>
     <row r="158" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>300</v>
@@ -11115,31 +11128,28 @@
         <v>282</v>
       </c>
       <c r="E158" t="s">
-        <v>642</v>
+        <v>637</v>
       </c>
       <c r="F158" t="s">
-        <v>643</v>
+        <v>638</v>
       </c>
       <c r="G158" t="s">
-        <v>644</v>
+        <v>639</v>
       </c>
       <c r="H158" t="s">
-        <v>645</v>
+        <v>640</v>
       </c>
       <c r="I158" t="s">
-        <v>646</v>
+        <v>641</v>
       </c>
       <c r="J158" s="9">
-        <v>5</v>
+        <v>3.8</v>
       </c>
       <c r="K158" s="15">
-        <v>330</v>
+        <v>200</v>
       </c>
       <c r="L158" t="s">
         <v>24</v>
-      </c>
-      <c r="M158" t="s">
-        <v>647</v>
       </c>
       <c r="N158" s="2" t="b">
         <v>0</v>
@@ -11159,7 +11169,7 @@
     </row>
     <row r="159" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="B159" s="2" t="s">
         <v>300</v>
@@ -11171,19 +11181,19 @@
         <v>282</v>
       </c>
       <c r="E159" t="s">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="F159" t="s">
-        <v>649</v>
+        <v>643</v>
       </c>
       <c r="G159" t="s">
-        <v>650</v>
+        <v>644</v>
       </c>
       <c r="H159" t="s">
-        <v>651</v>
+        <v>645</v>
       </c>
       <c r="I159" t="s">
-        <v>652</v>
+        <v>646</v>
       </c>
       <c r="J159" s="9">
         <v>5</v>
@@ -11194,6 +11204,9 @@
       <c r="L159" t="s">
         <v>24</v>
       </c>
+      <c r="M159" t="s">
+        <v>647</v>
+      </c>
       <c r="N159" s="2" t="b">
         <v>0</v>
       </c>
@@ -11212,7 +11225,7 @@
     </row>
     <row r="160" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="B160" s="2" t="s">
         <v>300</v>
@@ -11224,19 +11237,19 @@
         <v>282</v>
       </c>
       <c r="E160" t="s">
-        <v>653</v>
+        <v>648</v>
       </c>
       <c r="F160" t="s">
-        <v>654</v>
+        <v>649</v>
       </c>
       <c r="G160" t="s">
-        <v>655</v>
+        <v>650</v>
       </c>
       <c r="H160" t="s">
-        <v>656</v>
+        <v>651</v>
       </c>
       <c r="I160" t="s">
-        <v>657</v>
+        <v>652</v>
       </c>
       <c r="J160" s="9">
         <v>5</v>
@@ -11264,57 +11277,61 @@
       </c>
     </row>
     <row r="161" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A161" s="2" t="s">
+      <c r="A161" t="s">
+        <v>653</v>
+      </c>
+      <c r="B161" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C161" t="s">
+        <v>540</v>
+      </c>
+      <c r="D161" t="s">
+        <v>282</v>
+      </c>
+      <c r="E161" t="s">
+        <v>653</v>
+      </c>
+      <c r="F161" t="s">
+        <v>654</v>
+      </c>
+      <c r="G161" t="s">
+        <v>655</v>
+      </c>
+      <c r="H161" t="s">
+        <v>656</v>
+      </c>
+      <c r="I161" t="s">
+        <v>657</v>
+      </c>
+      <c r="J161" s="9">
+        <v>5</v>
+      </c>
+      <c r="K161" s="15">
+        <v>330</v>
+      </c>
+      <c r="L161" t="s">
+        <v>24</v>
+      </c>
+      <c r="N161" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O161" t="b">
+        <v>0</v>
+      </c>
+      <c r="P161" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q161" t="b">
+        <v>1</v>
+      </c>
+      <c r="R161" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="162" spans="1:19" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A162" s="2" t="s">
         <v>658</v>
-      </c>
-      <c r="B161" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C161" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="D161" s="2"/>
-      <c r="E161" s="2"/>
-      <c r="F161" s="2" t="s">
-        <v>659</v>
-      </c>
-      <c r="G161" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="H161" s="2"/>
-      <c r="I161" s="2"/>
-      <c r="J161" s="18">
-        <v>6</v>
-      </c>
-      <c r="K161" s="16">
-        <v>220</v>
-      </c>
-      <c r="L161" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M161" s="2"/>
-      <c r="N161" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O161" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P161" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q161" t="b">
-        <v>1</v>
-      </c>
-      <c r="R161" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S161" s="2">
-        <v>3.7</v>
-      </c>
-    </row>
-    <row r="162" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A162" s="2" t="s">
-        <v>661</v>
       </c>
       <c r="B162" s="2" t="s">
         <v>43</v>
@@ -11325,29 +11342,23 @@
       <c r="D162" s="2"/>
       <c r="E162" s="2"/>
       <c r="F162" s="2" t="s">
-        <v>662</v>
+        <v>659</v>
       </c>
       <c r="G162" s="2" t="s">
-        <v>663</v>
-      </c>
-      <c r="H162" s="2" t="s">
-        <v>664</v>
-      </c>
-      <c r="I162" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="J162" s="8">
+        <v>660</v>
+      </c>
+      <c r="H162" s="2"/>
+      <c r="I162" s="2"/>
+      <c r="J162" s="18">
         <v>6</v>
       </c>
       <c r="K162" s="16">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="L162" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M162" s="2" t="s">
-        <v>666</v>
-      </c>
+      <c r="M162" s="2"/>
       <c r="N162" s="2" t="b">
         <v>0</v>
       </c>
@@ -11363,45 +11374,45 @@
       <c r="R162" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="S162" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="163" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S162" s="2">
+        <v>3.7</v>
+      </c>
+    </row>
+    <row r="163" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
-        <v>668</v>
+        <v>661</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>669</v>
+        <v>292</v>
       </c>
       <c r="D163" s="2"/>
       <c r="E163" s="2"/>
       <c r="F163" s="2" t="s">
-        <v>670</v>
+        <v>662</v>
       </c>
       <c r="G163" s="2" t="s">
-        <v>671</v>
+        <v>663</v>
       </c>
       <c r="H163" s="2" t="s">
-        <v>672</v>
+        <v>664</v>
       </c>
       <c r="I163" s="2" t="s">
-        <v>673</v>
-      </c>
-      <c r="J163" s="18">
-        <v>8.5</v>
+        <v>665</v>
+      </c>
+      <c r="J163" s="8">
+        <v>6</v>
       </c>
       <c r="K163" s="16">
-        <v>330</v>
+        <v>300</v>
       </c>
       <c r="L163" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M163" s="2" t="s">
-        <v>674</v>
+        <v>666</v>
       </c>
       <c r="N163" s="2" t="b">
         <v>0</v>
@@ -11416,47 +11427,47 @@
         <v>1</v>
       </c>
       <c r="R163" s="2" t="s">
-        <v>675</v>
+        <v>297</v>
       </c>
       <c r="S163" s="2" t="s">
-        <v>667</v>
+        <v>447</v>
       </c>
     </row>
     <row r="164" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
-        <v>676</v>
+        <v>668</v>
       </c>
       <c r="B164" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>619</v>
+        <v>669</v>
       </c>
       <c r="D164" s="2"/>
       <c r="E164" s="2"/>
       <c r="F164" s="2" t="s">
-        <v>677</v>
+        <v>670</v>
       </c>
       <c r="G164" s="2" t="s">
-        <v>678</v>
+        <v>671</v>
       </c>
       <c r="H164" s="2" t="s">
-        <v>679</v>
+        <v>672</v>
       </c>
       <c r="I164" s="2" t="s">
-        <v>680</v>
-      </c>
-      <c r="J164" s="8">
-        <v>7.5</v>
+        <v>673</v>
+      </c>
+      <c r="J164" s="18">
+        <v>8.5</v>
       </c>
       <c r="K164" s="16">
-        <v>400</v>
+        <v>330</v>
       </c>
       <c r="L164" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M164" s="2" t="s">
-        <v>681</v>
+        <v>674</v>
       </c>
       <c r="N164" s="2" t="b">
         <v>0</v>
@@ -11471,47 +11482,47 @@
         <v>1</v>
       </c>
       <c r="R164" s="2" t="s">
-        <v>624</v>
+        <v>675</v>
       </c>
       <c r="S164" s="2" t="s">
-        <v>447</v>
-      </c>
-    </row>
-    <row r="165" spans="1:19" ht="138" customHeight="1" x14ac:dyDescent="0.3">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="165" spans="1:19" ht="96.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
-        <v>682</v>
+        <v>676</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>669</v>
+        <v>619</v>
       </c>
       <c r="D165" s="2"/>
       <c r="E165" s="2"/>
       <c r="F165" s="2" t="s">
-        <v>683</v>
+        <v>677</v>
       </c>
       <c r="G165" s="2" t="s">
-        <v>684</v>
+        <v>678</v>
       </c>
       <c r="H165" s="2" t="s">
-        <v>685</v>
+        <v>679</v>
       </c>
       <c r="I165" s="2" t="s">
-        <v>686</v>
-      </c>
-      <c r="J165" s="18">
-        <v>6.5</v>
+        <v>680</v>
+      </c>
+      <c r="J165" s="8">
+        <v>7.5</v>
       </c>
       <c r="K165" s="16">
-        <v>330</v>
+        <v>400</v>
       </c>
       <c r="L165" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M165" s="2" t="s">
-        <v>687</v>
+        <v>681</v>
       </c>
       <c r="N165" s="2" t="b">
         <v>0</v>
@@ -11526,47 +11537,47 @@
         <v>1</v>
       </c>
       <c r="R165" s="2" t="s">
-        <v>675</v>
+        <v>624</v>
       </c>
       <c r="S165" s="2" t="s">
-        <v>688</v>
-      </c>
-    </row>
-    <row r="166" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="166" spans="1:19" ht="138" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
-        <v>689</v>
+        <v>682</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>43</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>292</v>
+        <v>669</v>
       </c>
       <c r="D166" s="2"/>
       <c r="E166" s="2"/>
       <c r="F166" s="2" t="s">
-        <v>690</v>
+        <v>683</v>
       </c>
       <c r="G166" s="2" t="s">
-        <v>691</v>
+        <v>684</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>692</v>
+        <v>685</v>
       </c>
       <c r="I166" s="2" t="s">
-        <v>693</v>
-      </c>
-      <c r="J166" s="8">
-        <v>8</v>
+        <v>686</v>
+      </c>
+      <c r="J166" s="18">
+        <v>6.5</v>
       </c>
       <c r="K166" s="16">
-        <v>300</v>
+        <v>330</v>
       </c>
       <c r="L166" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M166" s="2" t="s">
-        <v>694</v>
+        <v>687</v>
       </c>
       <c r="N166" s="2" t="b">
         <v>0</v>
@@ -11581,15 +11592,15 @@
         <v>1</v>
       </c>
       <c r="R166" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="S166" s="2">
-        <v>7.8</v>
+        <v>675</v>
+      </c>
+      <c r="S166" s="2" t="s">
+        <v>688</v>
       </c>
     </row>
     <row r="167" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
-        <v>910</v>
+        <v>689</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>43</v>
@@ -11600,23 +11611,29 @@
       <c r="D167" s="2"/>
       <c r="E167" s="2"/>
       <c r="F167" s="2" t="s">
-        <v>911</v>
+        <v>690</v>
       </c>
       <c r="G167" s="2" t="s">
-        <v>912</v>
-      </c>
-      <c r="H167" s="2"/>
-      <c r="I167" s="2"/>
+        <v>691</v>
+      </c>
+      <c r="H167" s="2" t="s">
+        <v>692</v>
+      </c>
+      <c r="I167" s="2" t="s">
+        <v>693</v>
+      </c>
       <c r="J167" s="8">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K167" s="16">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="L167" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M167" s="2"/>
+      <c r="M167" s="2" t="s">
+        <v>694</v>
+      </c>
       <c r="N167" s="2" t="b">
         <v>0</v>
       </c>
@@ -11632,11 +11649,13 @@
       <c r="R167" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="S167" s="2"/>
-    </row>
-    <row r="168" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S167" s="2">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="168" spans="1:19" ht="69" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
-        <v>695</v>
+        <v>910</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>43</v>
@@ -11647,29 +11666,23 @@
       <c r="D168" s="2"/>
       <c r="E168" s="2"/>
       <c r="F168" s="2" t="s">
-        <v>696</v>
+        <v>911</v>
       </c>
       <c r="G168" s="2" t="s">
-        <v>697</v>
-      </c>
-      <c r="H168" s="2" t="s">
-        <v>698</v>
-      </c>
-      <c r="I168" s="2" t="s">
-        <v>699</v>
-      </c>
+        <v>912</v>
+      </c>
+      <c r="H168" s="2"/>
+      <c r="I168" s="2"/>
       <c r="J168" s="8">
-        <v>10.5</v>
+        <v>12</v>
       </c>
       <c r="K168" s="16">
-        <v>250</v>
+        <v>400</v>
       </c>
       <c r="L168" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M168" s="27" t="s">
-        <v>700</v>
-      </c>
+      <c r="M168" s="2"/>
       <c r="N168" s="2" t="b">
         <v>0</v>
       </c>
@@ -11685,60 +11698,66 @@
       <c r="R168" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="S168" s="2">
+      <c r="S168" s="2"/>
+    </row>
+    <row r="169" spans="1:19" ht="82.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A169" s="2" t="s">
+        <v>695</v>
+      </c>
+      <c r="B169" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C169" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D169" s="2"/>
+      <c r="E169" s="2"/>
+      <c r="F169" s="2" t="s">
+        <v>696</v>
+      </c>
+      <c r="G169" s="2" t="s">
+        <v>697</v>
+      </c>
+      <c r="H169" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="I169" s="2" t="s">
+        <v>699</v>
+      </c>
+      <c r="J169" s="8">
+        <v>10.5</v>
+      </c>
+      <c r="K169" s="16">
+        <v>250</v>
+      </c>
+      <c r="L169" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M169" s="27" t="s">
+        <v>700</v>
+      </c>
+      <c r="N169" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O169" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P169" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q169" t="b">
+        <v>1</v>
+      </c>
+      <c r="R169" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="S169" s="2">
         <v>7</v>
       </c>
     </row>
-    <row r="169" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
-      <c r="A169" t="s">
+    <row r="170" spans="1:19" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
         <v>701</v>
-      </c>
-      <c r="B169" t="s">
-        <v>20</v>
-      </c>
-      <c r="C169" s="21" t="s">
-        <v>526</v>
-      </c>
-      <c r="D169" t="s">
-        <v>527</v>
-      </c>
-      <c r="E169" t="s">
-        <v>528</v>
-      </c>
-      <c r="F169" t="s">
-        <v>702</v>
-      </c>
-      <c r="G169" t="s">
-        <v>703</v>
-      </c>
-      <c r="J169" s="9">
-        <v>13</v>
-      </c>
-      <c r="K169" s="15">
-        <v>750</v>
-      </c>
-      <c r="L169" t="s">
-        <v>24</v>
-      </c>
-      <c r="M169" s="2" t="s">
-        <v>833</v>
-      </c>
-      <c r="O169" t="b">
-        <v>0</v>
-      </c>
-      <c r="P169" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q169" t="b">
-        <v>1</v>
-      </c>
-      <c r="R169" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="170" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A170" t="s">
-        <v>704</v>
       </c>
       <c r="B170" t="s">
         <v>20</v>
@@ -11750,13 +11769,13 @@
         <v>527</v>
       </c>
       <c r="E170" t="s">
-        <v>532</v>
+        <v>528</v>
       </c>
       <c r="F170" t="s">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="G170" t="s">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="J170" s="9">
         <v>13</v>
@@ -11767,6 +11786,9 @@
       <c r="L170" t="s">
         <v>24</v>
       </c>
+      <c r="M170" s="2" t="s">
+        <v>833</v>
+      </c>
       <c r="O170" t="b">
         <v>0</v>
       </c>
@@ -11782,7 +11804,7 @@
     </row>
     <row r="171" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B171" t="s">
         <v>20</v>
@@ -11794,13 +11816,13 @@
         <v>527</v>
       </c>
       <c r="E171" t="s">
-        <v>536</v>
+        <v>532</v>
       </c>
       <c r="F171" t="s">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="G171" t="s">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="J171" s="9">
         <v>13</v>
@@ -11826,7 +11848,7 @@
     </row>
     <row r="172" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>855</v>
+        <v>707</v>
       </c>
       <c r="B172" t="s">
         <v>20</v>
@@ -11834,17 +11856,23 @@
       <c r="C172" s="21" t="s">
         <v>526</v>
       </c>
+      <c r="D172" t="s">
+        <v>527</v>
+      </c>
+      <c r="E172" t="s">
+        <v>536</v>
+      </c>
       <c r="F172" t="s">
-        <v>856</v>
+        <v>708</v>
       </c>
       <c r="G172" t="s">
-        <v>857</v>
+        <v>709</v>
       </c>
       <c r="J172" s="9">
-        <v>2.4</v>
+        <v>13</v>
       </c>
       <c r="K172" s="15">
-        <v>330</v>
+        <v>750</v>
       </c>
       <c r="L172" t="s">
         <v>24</v>
@@ -11862,113 +11890,96 @@
         <v>271</v>
       </c>
     </row>
-    <row r="173" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A173" s="2" t="s">
+    <row r="173" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>855</v>
+      </c>
+      <c r="B173" t="s">
+        <v>20</v>
+      </c>
+      <c r="C173" s="21" t="s">
+        <v>526</v>
+      </c>
+      <c r="F173" t="s">
+        <v>856</v>
+      </c>
+      <c r="G173" t="s">
+        <v>857</v>
+      </c>
+      <c r="J173" s="9">
+        <v>2.4</v>
+      </c>
+      <c r="K173" s="15">
+        <v>330</v>
+      </c>
+      <c r="L173" t="s">
+        <v>24</v>
+      </c>
+      <c r="O173" t="b">
+        <v>0</v>
+      </c>
+      <c r="P173" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q173" t="b">
+        <v>1</v>
+      </c>
+      <c r="R173" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="174" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A174" s="2" t="s">
         <v>710</v>
       </c>
-      <c r="B173" s="2" t="s">
+      <c r="B174" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C173" s="21" t="s">
+      <c r="C174" s="21" t="s">
         <v>65</v>
       </c>
-      <c r="D173" s="2" t="s">
+      <c r="D174" s="2" t="s">
         <v>711</v>
       </c>
-      <c r="E173" s="2" t="s">
+      <c r="E174" s="2" t="s">
         <v>712</v>
       </c>
-      <c r="F173" s="12" t="s">
+      <c r="F174" s="12" t="s">
         <v>713</v>
       </c>
-      <c r="G173" s="12" t="s">
+      <c r="G174" s="12" t="s">
         <v>714</v>
       </c>
-      <c r="H173" s="12"/>
-      <c r="I173" s="12"/>
-      <c r="J173" s="22"/>
-      <c r="K173" s="16">
+      <c r="H174" s="12"/>
+      <c r="I174" s="12"/>
+      <c r="J174" s="22"/>
+      <c r="K174" s="16">
         <v>50</v>
       </c>
-      <c r="L173" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M173" s="2"/>
-      <c r="N173" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O173" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P173" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q173" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="R173" s="2" t="s">
+      <c r="L174" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M174" s="2"/>
+      <c r="N174" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O174" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P174" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q174" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="R174" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="S173" s="2"/>
-    </row>
-    <row r="174" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A174" s="2" t="s">
-        <v>715</v>
-      </c>
-      <c r="B174" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>716</v>
-      </c>
-      <c r="D174" s="2"/>
-      <c r="E174" s="2"/>
-      <c r="F174" s="12" t="s">
-        <v>717</v>
-      </c>
-      <c r="G174" s="12" t="s">
-        <v>718</v>
-      </c>
-      <c r="H174" s="12" t="s">
-        <v>719</v>
-      </c>
-      <c r="I174" s="12" t="s">
-        <v>720</v>
-      </c>
-      <c r="J174" s="22">
-        <v>3.5</v>
-      </c>
-      <c r="K174" s="16">
-        <v>270</v>
-      </c>
-      <c r="L174" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="M174" s="2" t="s">
-        <v>721</v>
-      </c>
-      <c r="N174" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O174" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P174" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q174" t="b">
-        <v>1</v>
-      </c>
-      <c r="R174" s="2" t="s">
-        <v>722</v>
-      </c>
-      <c r="S174" s="2" t="s">
-        <v>447</v>
-      </c>
+      <c r="S174" s="2"/>
     </row>
     <row r="175" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
-        <v>723</v>
+        <v>715</v>
       </c>
       <c r="B175" s="2" t="s">
         <v>43</v>
@@ -11979,28 +11990,28 @@
       <c r="D175" s="2"/>
       <c r="E175" s="2"/>
       <c r="F175" s="12" t="s">
-        <v>724</v>
+        <v>717</v>
       </c>
       <c r="G175" s="12" t="s">
-        <v>725</v>
+        <v>718</v>
       </c>
       <c r="H175" s="12" t="s">
-        <v>726</v>
+        <v>719</v>
       </c>
       <c r="I175" s="12" t="s">
-        <v>727</v>
+        <v>720</v>
       </c>
       <c r="J175" s="22">
-        <v>8.5</v>
+        <v>3.5</v>
       </c>
       <c r="K175" s="16">
-        <v>300</v>
+        <v>270</v>
       </c>
       <c r="L175" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M175" s="2" t="s">
-        <v>728</v>
+        <v>721</v>
       </c>
       <c r="N175" s="2" t="b">
         <v>0</v>
@@ -12018,12 +12029,12 @@
         <v>722</v>
       </c>
       <c r="S175" s="2" t="s">
-        <v>729</v>
+        <v>447</v>
       </c>
     </row>
     <row r="176" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
-        <v>730</v>
+        <v>723</v>
       </c>
       <c r="B176" s="2" t="s">
         <v>43</v>
@@ -12034,28 +12045,28 @@
       <c r="D176" s="2"/>
       <c r="E176" s="2"/>
       <c r="F176" s="12" t="s">
-        <v>731</v>
+        <v>724</v>
       </c>
       <c r="G176" s="12" t="s">
-        <v>732</v>
+        <v>725</v>
       </c>
       <c r="H176" s="12" t="s">
-        <v>733</v>
+        <v>726</v>
       </c>
       <c r="I176" s="12" t="s">
-        <v>734</v>
+        <v>727</v>
       </c>
       <c r="J176" s="22">
-        <v>3.4</v>
+        <v>8.5</v>
       </c>
       <c r="K176" s="16">
-        <v>250</v>
+        <v>300</v>
       </c>
       <c r="L176" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M176" s="2" t="s">
-        <v>735</v>
+        <v>728</v>
       </c>
       <c r="N176" s="2" t="b">
         <v>0</v>
@@ -12073,12 +12084,12 @@
         <v>722</v>
       </c>
       <c r="S176" s="2" t="s">
-        <v>447</v>
+        <v>729</v>
       </c>
     </row>
     <row r="177" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
-        <v>736</v>
+        <v>730</v>
       </c>
       <c r="B177" s="2" t="s">
         <v>43</v>
@@ -12089,28 +12100,28 @@
       <c r="D177" s="2"/>
       <c r="E177" s="2"/>
       <c r="F177" s="12" t="s">
-        <v>737</v>
+        <v>731</v>
       </c>
       <c r="G177" s="12" t="s">
-        <v>738</v>
+        <v>732</v>
       </c>
       <c r="H177" s="12" t="s">
-        <v>739</v>
+        <v>733</v>
       </c>
       <c r="I177" s="12" t="s">
-        <v>740</v>
+        <v>734</v>
       </c>
       <c r="J177" s="22">
-        <v>3.1</v>
+        <v>3.4</v>
       </c>
       <c r="K177" s="16">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="L177" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M177" s="2" t="s">
-        <v>741</v>
+        <v>735</v>
       </c>
       <c r="N177" s="2" t="b">
         <v>0</v>
@@ -12127,13 +12138,13 @@
       <c r="R177" s="2" t="s">
         <v>722</v>
       </c>
-      <c r="S177" s="25" t="s">
-        <v>298</v>
+      <c r="S177" s="2" t="s">
+        <v>447</v>
       </c>
     </row>
     <row r="178" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
-        <v>742</v>
+        <v>736</v>
       </c>
       <c r="B178" s="2" t="s">
         <v>43</v>
@@ -12144,28 +12155,28 @@
       <c r="D178" s="2"/>
       <c r="E178" s="2"/>
       <c r="F178" s="12" t="s">
-        <v>743</v>
+        <v>737</v>
       </c>
       <c r="G178" s="12" t="s">
-        <v>744</v>
+        <v>738</v>
       </c>
       <c r="H178" s="12" t="s">
-        <v>745</v>
+        <v>739</v>
       </c>
       <c r="I178" s="12" t="s">
-        <v>746</v>
+        <v>740</v>
       </c>
       <c r="J178" s="22">
-        <v>6</v>
+        <v>3.1</v>
       </c>
       <c r="K178" s="16">
-        <v>270</v>
+        <v>400</v>
       </c>
       <c r="L178" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M178" s="2" t="s">
-        <v>747</v>
+        <v>741</v>
       </c>
       <c r="N178" s="2" t="b">
         <v>0</v>
@@ -12183,12 +12194,12 @@
         <v>722</v>
       </c>
       <c r="S178" s="25" t="s">
-        <v>628</v>
+        <v>298</v>
       </c>
     </row>
     <row r="179" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
-        <v>748</v>
+        <v>742</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>43</v>
@@ -12199,22 +12210,28 @@
       <c r="D179" s="2"/>
       <c r="E179" s="2"/>
       <c r="F179" s="12" t="s">
-        <v>749</v>
+        <v>743</v>
       </c>
       <c r="G179" s="12" t="s">
-        <v>750</v>
-      </c>
-      <c r="H179" s="12"/>
-      <c r="I179" s="12"/>
+        <v>744</v>
+      </c>
+      <c r="H179" s="12" t="s">
+        <v>745</v>
+      </c>
+      <c r="I179" s="12" t="s">
+        <v>746</v>
+      </c>
       <c r="J179" s="22">
-        <v>7.5</v>
-      </c>
-      <c r="K179" s="16"/>
+        <v>6</v>
+      </c>
+      <c r="K179" s="16">
+        <v>270</v>
+      </c>
       <c r="L179" s="2" t="s">
         <v>57</v>
       </c>
       <c r="M179" s="2" t="s">
-        <v>751</v>
+        <v>747</v>
       </c>
       <c r="N179" s="2" t="b">
         <v>0</v>
@@ -12232,121 +12249,129 @@
         <v>722</v>
       </c>
       <c r="S179" s="25" t="s">
-        <v>752</v>
-      </c>
-    </row>
-    <row r="180" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="180" spans="1:19" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>300</v>
+        <v>43</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>301</v>
+        <v>716</v>
       </c>
       <c r="D180" s="2"/>
       <c r="E180" s="2"/>
       <c r="F180" s="12" t="s">
+        <v>749</v>
+      </c>
+      <c r="G180" s="12" t="s">
+        <v>750</v>
+      </c>
+      <c r="H180" s="12"/>
+      <c r="I180" s="12"/>
+      <c r="J180" s="22">
+        <v>7.5</v>
+      </c>
+      <c r="K180" s="16"/>
+      <c r="L180" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M180" s="2" t="s">
+        <v>751</v>
+      </c>
+      <c r="N180" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O180" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P180" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q180" t="b">
+        <v>1</v>
+      </c>
+      <c r="R180" s="2" t="s">
+        <v>722</v>
+      </c>
+      <c r="S180" s="25" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="181" spans="1:19" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="2" t="s">
+        <v>753</v>
+      </c>
+      <c r="B181" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C181" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="D181" s="2"/>
+      <c r="E181" s="2"/>
+      <c r="F181" s="12" t="s">
         <v>754</v>
       </c>
-      <c r="G180" s="12" t="s">
+      <c r="G181" s="12" t="s">
         <v>755</v>
       </c>
-      <c r="H180" s="12" t="s">
+      <c r="H181" s="12" t="s">
         <v>756</v>
       </c>
-      <c r="I180" s="12" t="s">
+      <c r="I181" s="12" t="s">
         <v>757</v>
       </c>
-      <c r="J180" s="22">
+      <c r="J181" s="22">
         <v>3.5</v>
       </c>
-      <c r="K180" s="20">
+      <c r="K181" s="20">
         <v>150</v>
       </c>
-      <c r="L180" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M180" s="2"/>
-      <c r="N180" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="O180" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="P180" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q180" t="b">
-        <v>1</v>
-      </c>
-      <c r="R180" s="2" t="s">
+      <c r="L181" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M181" s="2"/>
+      <c r="N181" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O181" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="P181" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q181" t="b">
+        <v>1</v>
+      </c>
+      <c r="R181" s="2" t="s">
         <v>758</v>
       </c>
-      <c r="S180" s="2"/>
-    </row>
-    <row r="181" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A181" t="s">
-        <v>759</v>
-      </c>
-      <c r="B181" t="s">
-        <v>20</v>
-      </c>
-      <c r="C181" s="21" t="s">
-        <v>21</v>
-      </c>
-      <c r="F181" s="13" t="s">
-        <v>760</v>
-      </c>
-      <c r="G181" s="13" t="s">
-        <v>761</v>
-      </c>
-      <c r="H181" s="13"/>
-      <c r="I181" s="13"/>
-      <c r="J181" s="22">
-        <v>3.1</v>
-      </c>
-      <c r="K181" s="15"/>
-      <c r="L181" t="s">
-        <v>24</v>
-      </c>
-      <c r="N181" t="b">
-        <v>0</v>
-      </c>
-      <c r="O181" t="b">
-        <v>0</v>
-      </c>
-      <c r="P181" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q181" t="b">
-        <v>1</v>
-      </c>
-      <c r="R181" t="s">
-        <v>25</v>
-      </c>
+      <c r="S181" s="2"/>
     </row>
     <row r="182" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>762</v>
+        <v>759</v>
       </c>
       <c r="B182" t="s">
         <v>20</v>
       </c>
       <c r="C182" s="21" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="F182" s="13" t="s">
-        <v>763</v>
+        <v>760</v>
       </c>
       <c r="G182" s="13" t="s">
-        <v>764</v>
+        <v>761</v>
       </c>
       <c r="H182" s="13"/>
       <c r="I182" s="13"/>
       <c r="J182" s="22">
-        <v>1.8</v>
+        <v>3.1</v>
       </c>
       <c r="K182" s="15"/>
       <c r="L182" t="s">
@@ -12370,7 +12395,7 @@
     </row>
     <row r="183" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="B183" t="s">
         <v>20</v>
@@ -12378,18 +12403,21 @@
       <c r="C183" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="F183" s="14" t="s">
-        <v>766</v>
+      <c r="F183" s="13" t="s">
+        <v>763</v>
       </c>
       <c r="G183" s="13" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="H183" s="13"/>
       <c r="I183" s="13"/>
       <c r="J183" s="22">
-        <v>0.4</v>
+        <v>1.8</v>
       </c>
       <c r="K183" s="15"/>
+      <c r="L183" t="s">
+        <v>24</v>
+      </c>
       <c r="N183" t="b">
         <v>0</v>
       </c>
@@ -12408,34 +12436,26 @@
     </row>
     <row r="184" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
-        <v>768</v>
+        <v>765</v>
       </c>
       <c r="B184" t="s">
         <v>20</v>
       </c>
-      <c r="C184" t="s">
-        <v>60</v>
-      </c>
-      <c r="D184" t="s">
-        <v>120</v>
-      </c>
-      <c r="F184" s="13" t="s">
-        <v>121</v>
+      <c r="C184" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F184" s="14" t="s">
+        <v>766</v>
       </c>
       <c r="G184" s="13" t="s">
-        <v>122</v>
+        <v>767</v>
       </c>
       <c r="H184" s="13"/>
       <c r="I184" s="13"/>
       <c r="J184" s="22">
-        <v>1.2</v>
-      </c>
-      <c r="K184" s="15">
-        <v>500</v>
-      </c>
-      <c r="L184" t="s">
-        <v>24</v>
-      </c>
+        <v>0.4</v>
+      </c>
+      <c r="K184" s="15"/>
       <c r="N184" t="b">
         <v>0</v>
       </c>
@@ -12454,7 +12474,7 @@
     </row>
     <row r="185" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B185" t="s">
         <v>20</v>
@@ -12462,19 +12482,22 @@
       <c r="C185" t="s">
         <v>60</v>
       </c>
+      <c r="D185" t="s">
+        <v>120</v>
+      </c>
       <c r="F185" s="13" t="s">
-        <v>770</v>
+        <v>121</v>
       </c>
       <c r="G185" s="13" t="s">
-        <v>771</v>
+        <v>122</v>
       </c>
       <c r="H185" s="13"/>
       <c r="I185" s="13"/>
       <c r="J185" s="22">
-        <v>4.0999999999999996</v>
+        <v>1.2</v>
       </c>
       <c r="K185" s="15">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="L185" t="s">
         <v>24</v>
@@ -12495,8 +12518,51 @@
         <v>25</v>
       </c>
     </row>
+    <row r="186" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>769</v>
+      </c>
+      <c r="B186" t="s">
+        <v>20</v>
+      </c>
+      <c r="C186" t="s">
+        <v>60</v>
+      </c>
+      <c r="F186" s="13" t="s">
+        <v>770</v>
+      </c>
+      <c r="G186" s="13" t="s">
+        <v>771</v>
+      </c>
+      <c r="H186" s="13"/>
+      <c r="I186" s="13"/>
+      <c r="J186" s="22">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="K186" s="15">
+        <v>200</v>
+      </c>
+      <c r="L186" t="s">
+        <v>24</v>
+      </c>
+      <c r="N186" t="b">
+        <v>0</v>
+      </c>
+      <c r="O186" t="b">
+        <v>0</v>
+      </c>
+      <c r="P186" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q186" t="b">
+        <v>1</v>
+      </c>
+      <c r="R186" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S121"/>
+  <autoFilter ref="A1:S122"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>